<commit_message>
Add mobile equipment fleet (16 items) and full staffing roster (34 positions, 67 headcount) to CAPEX_OPEX tab
- MOBILE EQUIPMENT section: loaders, trucks, forklifts, trailers, attachments (~$685k)
- STAFFING section: all 34 positions with headcount, salary, shift pattern, monthly cost formulas
- OPEX labour line now formula-linked to staffing total (=E156) instead of hardcoded estimate
- Column widths expanded to accommodate staffing detail (6 columns)
- No employee/HR tables found in SQL migrations — staffing based on Indonesian palm sector averages

https://claude.ai/code/session_01WZKNxbjsTJxtui6XGx7d89
</commit_message>
<xml_diff>
--- a/CFI_Master_Excel.xlsx
+++ b/CFI_Master_Excel.xlsx
@@ -248,7 +248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -349,6 +349,13 @@
     </xf>
     <xf numFmtId="167" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -4542,13 +4549,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D123"/>
+  <dimension ref="A1:F183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5861,285 +5870,1562 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>TOTAL CAPEX SUMMARY</t>
+          <t>MOBILE EQUIPMENT &amp; VEHICLES</t>
         </is>
       </c>
       <c r="B99" s="3" t="n"/>
       <c r="C99" s="3" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="38" t="inlineStr">
-        <is>
-          <t>TOTAL CAPEX</t>
-        </is>
-      </c>
-      <c r="B100" s="51">
-        <f>IFERROR(SUM(B5:B99),0)</f>
-        <v/>
+      <c r="A100" s="9" t="inlineStr">
+        <is>
+          <t>Equipment / Item</t>
+        </is>
+      </c>
+      <c r="B100" s="9" t="inlineStr">
+        <is>
+          <t>Estimated Cost (USD)</t>
+        </is>
+      </c>
+      <c r="C100" s="9" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="10" t="inlineStr">
+        <is>
+          <t>Wheel Loader — Komatsu WA100 or equiv (1.0m3 bucket, EFB/OPDC handling)</t>
+        </is>
+      </c>
+      <c r="B101" s="46" t="n">
+        <v>85000</v>
+      </c>
+      <c r="C101" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="3" t="inlineStr">
-        <is>
-          <t>MONTHLY OPERATING EXPENDITURE (OPEX)</t>
-        </is>
-      </c>
-      <c r="B102" s="3" t="n"/>
-      <c r="C102" s="3" t="n"/>
-      <c r="D102" s="3" t="n"/>
+      <c r="A102" s="10" t="inlineStr">
+        <is>
+          <t>Wheel Loader — Komatsu WA70 or equiv (0.5m3 bucket, PKSA/compost)</t>
+        </is>
+      </c>
+      <c r="B102" s="46" t="n">
+        <v>55000</v>
+      </c>
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="9" t="inlineStr">
-        <is>
-          <t>Cost Item</t>
-        </is>
-      </c>
-      <c r="B103" s="9" t="inlineStr">
-        <is>
-          <t>Monthly Cost (USD)</t>
-        </is>
-      </c>
-      <c r="C103" s="9" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A103" s="10" t="inlineStr">
+        <is>
+          <t>Skid-Steer Loader / Bobcat — S650 or equiv (BSF frass, substrate)</t>
+        </is>
+      </c>
+      <c r="B103" s="46" t="n">
+        <v>45000</v>
+      </c>
+      <c r="C103" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>Chemical Treatment</t>
-        </is>
-      </c>
-      <c r="B104" s="22">
-        <f>IFERROR(S2_Chemical_Treatment!B33,0)</f>
-        <v/>
-      </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>From Stage 2</t>
+          <t>Skid-Steer Loader / Bobcat — S450 or equiv (greenhouse internal)</t>
+        </is>
+      </c>
+      <c r="B104" s="46" t="n">
+        <v>38000</v>
+      </c>
+      <c r="C104" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Biological Treatment</t>
-        </is>
-      </c>
-      <c r="B105" s="22">
-        <f>IFERROR(S3_Biological_Treatment!B33,0)</f>
-        <v/>
-      </c>
-      <c r="C105" s="2" t="inlineStr">
-        <is>
-          <t>From Stage 3</t>
+          <t>Mini Excavator — 3.5t (site maintenance, drainage, pit cleaning)</t>
+        </is>
+      </c>
+      <c r="B105" s="46" t="n">
+        <v>42000</v>
+      </c>
+      <c r="C105" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>BSF Neonates</t>
-        </is>
-      </c>
-      <c r="B106" s="22">
-        <f>IFERROR(S4_BSF_Rearing!B8,0)</f>
-        <v/>
-      </c>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t>From Stage 4</t>
+          <t>Dump Truck — 10t (EFB transport mill to S1, internal)</t>
+        </is>
+      </c>
+      <c r="B106" s="46" t="n">
+        <v>65000</v>
+      </c>
+      <c r="C106" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>Processing (S5B)</t>
-        </is>
-      </c>
-      <c r="B107" s="22">
-        <f>IFERROR(S5B_BSF_Extraction!B29,0)</f>
-        <v/>
-      </c>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t>From Stage 5B</t>
+          <t>Dump Truck — 10t (OPDC/POS transport mill to S1)</t>
+        </is>
+      </c>
+      <c r="B107" s="46" t="n">
+        <v>65000</v>
+      </c>
+      <c r="C107" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
         <is>
-          <t>Energy / Utilities</t>
-        </is>
-      </c>
-      <c r="B108" s="22">
-        <f>IFERROR(S1_Preprocessing!B30,0)</f>
-        <v/>
-      </c>
-      <c r="C108" s="2" t="inlineStr">
-        <is>
-          <t>From Stage 1</t>
+          <t>Flatbed Truck — 8t (finished product transport, frass/meal)</t>
+        </is>
+      </c>
+      <c r="B108" s="46" t="n">
+        <v>55000</v>
+      </c>
+      <c r="C108" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>Labour (estimated)</t>
+          <t>Tanker Truck — 5,000L (water, POME, liquid transfer)</t>
         </is>
       </c>
       <c r="B109" s="46" t="n">
-        <v>8000</v>
-      </c>
-      <c r="C109" s="2" t="inlineStr">
-        <is>
-          <t>10 workers @ $800/month</t>
+        <v>48000</v>
+      </c>
+      <c r="C109" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
         <is>
-          <t>Maintenance (2% CAPEX/month)</t>
-        </is>
-      </c>
-      <c r="B110" s="22">
-        <f>IFERROR(B100*0.02/12,0)</f>
-        <v/>
-      </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>Industry standard</t>
+          <t>Pickup Truck — 4x4 (site management, 2 units)</t>
+        </is>
+      </c>
+      <c r="B110" s="46" t="n">
+        <v>60000</v>
+      </c>
+      <c r="C110" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>Quality Control / Lab</t>
+          <t>Forklift — 3t diesel (warehouse, bagged product, 2 units)</t>
         </is>
       </c>
       <c r="B111" s="46" t="n">
-        <v>2000</v>
-      </c>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>Monthly QC testing</t>
+        <v>50000</v>
+      </c>
+      <c r="C111" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
         <is>
+          <t>Forklift — 1.5t electric (greenhouse internal, 2 units)</t>
+        </is>
+      </c>
+      <c r="B112" s="46" t="n">
+        <v>36000</v>
+      </c>
+      <c r="C112" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="10" t="inlineStr">
+        <is>
+          <t>Tipping Trailer — 8t (substrate/frass haulage, 2 units)</t>
+        </is>
+      </c>
+      <c r="B113" s="46" t="n">
+        <v>24000</v>
+      </c>
+      <c r="C113" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="10" t="inlineStr">
+        <is>
+          <t>Pallet Jacks — manual (4 units, warehouse)</t>
+        </is>
+      </c>
+      <c r="B114" s="46" t="n">
+        <v>3200</v>
+      </c>
+      <c r="C114" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>Grab Bucket Attachment — for wheel loader (EFB)</t>
+        </is>
+      </c>
+      <c r="B115" s="46" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C115" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="10" t="inlineStr">
+        <is>
+          <t>Sweeper Attachment — for bobcat (greenhouse cleaning)</t>
+        </is>
+      </c>
+      <c r="B116" s="46" t="n">
+        <v>6500</v>
+      </c>
+      <c r="C116" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="7" t="inlineStr">
+        <is>
+          <t>Mobile Equipment Subtotal</t>
+        </is>
+      </c>
+      <c r="B117" s="22">
+        <f>SUM(B101:B116)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>STAFFING — FULL HEADCOUNT &amp; LABOUR COST</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="n"/>
+      <c r="C119" s="3" t="n"/>
+      <c r="D119" s="3" t="n"/>
+      <c r="E119" s="3" t="n"/>
+      <c r="F119" s="3" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="9" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="B120" s="9" t="inlineStr">
+        <is>
+          <t>Headcount</t>
+        </is>
+      </c>
+      <c r="C120" s="9" t="inlineStr">
+        <is>
+          <t>Salary (USD/month)</t>
+        </is>
+      </c>
+      <c r="D120" s="9" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="E120" s="9" t="inlineStr">
+        <is>
+          <t>Monthly Cost (USD)</t>
+        </is>
+      </c>
+      <c r="F120" s="9" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="10" t="inlineStr">
+        <is>
+          <t>S1 — EFB Line Operator (shredder + hammer mill)</t>
+        </is>
+      </c>
+      <c r="B121" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C121" s="46" t="n">
+        <v>450</v>
+      </c>
+      <c r="D121" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E121" s="22">
+        <f>B121*C121</f>
+        <v/>
+      </c>
+      <c r="F121" s="54" t="inlineStr">
+        <is>
+          <t>1 per shift, monitors feed + oversize return</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="10" t="inlineStr">
+        <is>
+          <t>S1 — EFB Conveyor / Screen Operator</t>
+        </is>
+      </c>
+      <c r="B122" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C122" s="46" t="n">
+        <v>400</v>
+      </c>
+      <c r="D122" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E122" s="22">
+        <f>B122*C122</f>
+        <v/>
+      </c>
+      <c r="F122" s="54" t="inlineStr">
+        <is>
+          <t>Belt + vibrating screen monitoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="10" t="inlineStr">
+        <is>
+          <t>S1 — EFB Screw Press Operator</t>
+        </is>
+      </c>
+      <c r="B123" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C123" s="46" t="n">
+        <v>450</v>
+      </c>
+      <c r="D123" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E123" s="22">
+        <f>B123*C123</f>
+        <v/>
+      </c>
+      <c r="F123" s="54" t="inlineStr">
+        <is>
+          <t>MC control, filtrate routing</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="inlineStr">
+        <is>
+          <t>S1 — OPDC Line Operator (shredder + hammer mill)</t>
+        </is>
+      </c>
+      <c r="B124" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C124" s="46" t="n">
+        <v>450</v>
+      </c>
+      <c r="D124" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E124" s="22">
+        <f>B124*C124</f>
+        <v/>
+      </c>
+      <c r="F124" s="54" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="10" t="inlineStr">
+        <is>
+          <t>S1 — OPDC Conveyor / Press Operator</t>
+        </is>
+      </c>
+      <c r="B125" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C125" s="46" t="n">
+        <v>400</v>
+      </c>
+      <c r="D125" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E125" s="22">
+        <f>B125*C125</f>
+        <v/>
+      </c>
+      <c r="F125" s="54" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="10" t="inlineStr">
+        <is>
+          <t>S1 — POS Decanter Operator</t>
+        </is>
+      </c>
+      <c r="B126" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C126" s="46" t="n">
+        <v>550</v>
+      </c>
+      <c r="D126" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E126" s="22">
+        <f>B126*C126</f>
+        <v/>
+      </c>
+      <c r="F126" s="54" t="inlineStr">
+        <is>
+          <t>Skilled: centrifuge operation + Fe gate sampling</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="10" t="inlineStr">
+        <is>
+          <t>S1 — Wheel Loader Operator (EFB/OPDC feed)</t>
+        </is>
+      </c>
+      <c r="B127" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C127" s="46" t="n">
+        <v>500</v>
+      </c>
+      <c r="D127" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E127" s="22">
+        <f>B127*C127</f>
+        <v/>
+      </c>
+      <c r="F127" s="54" t="inlineStr">
+        <is>
+          <t>Komatsu WA100</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="10" t="inlineStr">
+        <is>
+          <t>S1 — Dump Truck Driver (mill to S1)</t>
+        </is>
+      </c>
+      <c r="B128" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C128" s="46" t="n">
+        <v>450</v>
+      </c>
+      <c r="D128" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E128" s="22">
+        <f>B128*C128</f>
+        <v/>
+      </c>
+      <c r="F128" s="54" t="inlineStr">
+        <is>
+          <t>2x 10t dump trucks</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="10" t="inlineStr">
+        <is>
+          <t>S2 — Chemical Dosing Operator</t>
+        </is>
+      </c>
+      <c r="B129" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C129" s="46" t="n">
+        <v>500</v>
+      </c>
+      <c r="D129" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E129" s="22">
+        <f>B129*C129</f>
+        <v/>
+      </c>
+      <c r="F129" s="54" t="inlineStr">
+        <is>
+          <t>PKSA/chemical mixing, pH monitoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="10" t="inlineStr">
+        <is>
+          <t>S2 — Neutralisation Bay Attendant</t>
+        </is>
+      </c>
+      <c r="B130" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C130" s="46" t="n">
+        <v>400</v>
+      </c>
+      <c r="D130" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E130" s="22">
+        <f>B130*C130</f>
+        <v/>
+      </c>
+      <c r="F130" s="54" t="inlineStr">
+        <is>
+          <t>Turnings at 8-12hr and 16-20hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="10" t="inlineStr">
+        <is>
+          <t>S3 — Biological Inoculation Technician</t>
+        </is>
+      </c>
+      <c r="B131" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C131" s="46" t="n">
+        <v>600</v>
+      </c>
+      <c r="D131" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E131" s="22">
+        <f>B131*C131</f>
+        <v/>
+      </c>
+      <c r="F131" s="54" t="inlineStr">
+        <is>
+          <t>Consortium preparation, spray application</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="10" t="inlineStr">
+        <is>
+          <t>S3 — Composting / Windrow Operator</t>
+        </is>
+      </c>
+      <c r="B132" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C132" s="46" t="n">
+        <v>450</v>
+      </c>
+      <c r="D132" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E132" s="22">
+        <f>B132*C132</f>
+        <v/>
+      </c>
+      <c r="F132" s="54" t="inlineStr">
+        <is>
+          <t>Windrow turner + aeration monitoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="10" t="inlineStr">
+        <is>
+          <t>S3 — Bobcat Operator (substrate handling)</t>
+        </is>
+      </c>
+      <c r="B133" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C133" s="46" t="n">
+        <v>450</v>
+      </c>
+      <c r="D133" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E133" s="22">
+        <f>B133*C133</f>
+        <v/>
+      </c>
+      <c r="F133" s="54" t="inlineStr">
+        <is>
+          <t>S650 skid-steer</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="10" t="inlineStr">
+        <is>
+          <t>S4 — Greenhouse Supervisor</t>
+        </is>
+      </c>
+      <c r="B134" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C134" s="46" t="n">
+        <v>900</v>
+      </c>
+      <c r="D134" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E134" s="22">
+        <f>B134*C134</f>
+        <v/>
+      </c>
+      <c r="F134" s="54" t="inlineStr">
+        <is>
+          <t>Overall BSF rearing management</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="10" t="inlineStr">
+        <is>
+          <t>S4 — BSF Tray Attendant (feeding + monitoring)</t>
+        </is>
+      </c>
+      <c r="B135" s="53" t="n">
+        <v>8</v>
+      </c>
+      <c r="C135" s="46" t="n">
+        <v>400</v>
+      </c>
+      <c r="D135" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E135" s="22">
+        <f>B135*C135</f>
+        <v/>
+      </c>
+      <c r="F135" s="54" t="inlineStr">
+        <is>
+          <t>4 per shift, 5000m2 per attendant</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="10" t="inlineStr">
+        <is>
+          <t>S4 — BSF Neonate Nursery Technician</t>
+        </is>
+      </c>
+      <c r="B136" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C136" s="46" t="n">
+        <v>550</v>
+      </c>
+      <c r="D136" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E136" s="22">
+        <f>B136*C136</f>
+        <v/>
+      </c>
+      <c r="F136" s="54" t="inlineStr">
+        <is>
+          <t>Colony management, egg collection</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="10" t="inlineStr">
+        <is>
+          <t>S4 — Greenhouse Climate / IoT Technician</t>
+        </is>
+      </c>
+      <c r="B137" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C137" s="46" t="n">
+        <v>700</v>
+      </c>
+      <c r="D137" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E137" s="22">
+        <f>B137*C137</f>
+        <v/>
+      </c>
+      <c r="F137" s="54" t="inlineStr">
+        <is>
+          <t>SCADA/PLC, sensor maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="10" t="inlineStr">
+        <is>
+          <t>S4 — Bobcat Operator (greenhouse internal)</t>
+        </is>
+      </c>
+      <c r="B138" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C138" s="46" t="n">
+        <v>450</v>
+      </c>
+      <c r="D138" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E138" s="22">
+        <f>B138*C138</f>
+        <v/>
+      </c>
+      <c r="F138" s="54" t="inlineStr">
+        <is>
+          <t>S450, substrate + frass movement</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="10" t="inlineStr">
+        <is>
+          <t>S4 — Forklift Operator (greenhouse)</t>
+        </is>
+      </c>
+      <c r="B139" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C139" s="46" t="n">
+        <v>400</v>
+      </c>
+      <c r="D139" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E139" s="22">
+        <f>B139*C139</f>
+        <v/>
+      </c>
+      <c r="F139" s="54" t="inlineStr">
+        <is>
+          <t>1.5t electric forklifts</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="10" t="inlineStr">
+        <is>
+          <t>S5A — Frass Screening / Bagging Operator</t>
+        </is>
+      </c>
+      <c r="B140" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C140" s="46" t="n">
+        <v>400</v>
+      </c>
+      <c r="D140" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E140" s="22">
+        <f>B140*C140</f>
+        <v/>
+      </c>
+      <c r="F140" s="54" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="10" t="inlineStr">
+        <is>
+          <t>S5B — Larvae Separation Operator</t>
+        </is>
+      </c>
+      <c r="B141" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C141" s="46" t="n">
+        <v>450</v>
+      </c>
+      <c r="D141" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E141" s="22">
+        <f>B141*C141</f>
+        <v/>
+      </c>
+      <c r="F141" s="54" t="inlineStr">
+        <is>
+          <t>Vibrating separator + thermal</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="10" t="inlineStr">
+        <is>
+          <t>S5B — Oil Press / Dryer Operator</t>
+        </is>
+      </c>
+      <c r="B142" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C142" s="46" t="n">
+        <v>500</v>
+      </c>
+      <c r="D142" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E142" s="22">
+        <f>B142*C142</f>
+        <v/>
+      </c>
+      <c r="F142" s="54" t="inlineStr">
+        <is>
+          <t>Screw press + belt dryer</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="10" t="inlineStr">
+        <is>
+          <t>Warehouse — Forklift Operator</t>
+        </is>
+      </c>
+      <c r="B143" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C143" s="46" t="n">
+        <v>400</v>
+      </c>
+      <c r="D143" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E143" s="22">
+        <f>B143*C143</f>
+        <v/>
+      </c>
+      <c r="F143" s="54" t="inlineStr">
+        <is>
+          <t>3t diesel forklift</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="10" t="inlineStr">
+        <is>
+          <t>Warehouse — Storeman / Inventory</t>
+        </is>
+      </c>
+      <c r="B144" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C144" s="46" t="n">
+        <v>450</v>
+      </c>
+      <c r="D144" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E144" s="22">
+        <f>B144*C144</f>
+        <v/>
+      </c>
+      <c r="F144" s="54" t="inlineStr">
+        <is>
+          <t>Stock control, dispatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="10" t="inlineStr">
+        <is>
+          <t>Logistics — Flatbed Truck Driver</t>
+        </is>
+      </c>
+      <c r="B145" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C145" s="46" t="n">
+        <v>450</v>
+      </c>
+      <c r="D145" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E145" s="22">
+        <f>B145*C145</f>
+        <v/>
+      </c>
+      <c r="F145" s="54" t="inlineStr">
+        <is>
+          <t>Product delivery</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="10" t="inlineStr">
+        <is>
+          <t>Logistics — Tanker Truck Driver</t>
+        </is>
+      </c>
+      <c r="B146" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C146" s="46" t="n">
+        <v>450</v>
+      </c>
+      <c r="D146" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E146" s="22">
+        <f>B146*C146</f>
+        <v/>
+      </c>
+      <c r="F146" s="54" t="inlineStr">
+        <is>
+          <t>Water/POME</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="10" t="inlineStr">
+        <is>
+          <t>Site Manager</t>
+        </is>
+      </c>
+      <c r="B147" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C147" s="46" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D147" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E147" s="22">
+        <f>B147*C147</f>
+        <v/>
+      </c>
+      <c r="F147" s="54" t="inlineStr">
+        <is>
+          <t>Overall plant management</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="10" t="inlineStr">
+        <is>
+          <t>Production Supervisor (S1-S3)</t>
+        </is>
+      </c>
+      <c r="B148" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C148" s="46" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D148" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E148" s="22">
+        <f>B148*C148</f>
+        <v/>
+      </c>
+      <c r="F148" s="54" t="inlineStr">
+        <is>
+          <t>Preprocessing + treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="10" t="inlineStr">
+        <is>
+          <t>Quality Control / Lab Technician</t>
+        </is>
+      </c>
+      <c r="B149" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C149" s="46" t="n">
+        <v>650</v>
+      </c>
+      <c r="D149" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E149" s="22">
+        <f>B149*C149</f>
+        <v/>
+      </c>
+      <c r="F149" s="54" t="inlineStr">
+        <is>
+          <t>pH, MC, ICP-OES, sampling</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="10" t="inlineStr">
+        <is>
+          <t>Maintenance Technician (mechanical)</t>
+        </is>
+      </c>
+      <c r="B150" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C150" s="46" t="n">
+        <v>600</v>
+      </c>
+      <c r="D150" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E150" s="22">
+        <f>B150*C150</f>
+        <v/>
+      </c>
+      <c r="F150" s="54" t="inlineStr">
+        <is>
+          <t>All mechanical equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="10" t="inlineStr">
+        <is>
+          <t>Maintenance Technician (electrical/IoT)</t>
+        </is>
+      </c>
+      <c r="B151" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C151" s="46" t="n">
+        <v>650</v>
+      </c>
+      <c r="D151" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E151" s="22">
+        <f>B151*C151</f>
+        <v/>
+      </c>
+      <c r="F151" s="54" t="inlineStr">
+        <is>
+          <t>Electrical, sensors, PLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="10" t="inlineStr">
+        <is>
+          <t>HSE Officer</t>
+        </is>
+      </c>
+      <c r="B152" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" s="46" t="n">
+        <v>700</v>
+      </c>
+      <c r="D152" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E152" s="22">
+        <f>B152*C152</f>
+        <v/>
+      </c>
+      <c r="F152" s="54" t="inlineStr">
+        <is>
+          <t>Safety, PPE, NaOH handling</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="10" t="inlineStr">
+        <is>
+          <t>Admin / Finance</t>
+        </is>
+      </c>
+      <c r="B153" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C153" s="46" t="n">
+        <v>500</v>
+      </c>
+      <c r="D153" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E153" s="22">
+        <f>B153*C153</f>
+        <v/>
+      </c>
+      <c r="F153" s="54" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="10" t="inlineStr">
+        <is>
+          <t>Security (gate + night)</t>
+        </is>
+      </c>
+      <c r="B154" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="C154" s="46" t="n">
+        <v>350</v>
+      </c>
+      <c r="D154" s="53" t="inlineStr">
+        <is>
+          <t>3-shift</t>
+        </is>
+      </c>
+      <c r="E154" s="22">
+        <f>B154*C154</f>
+        <v/>
+      </c>
+      <c r="F154" s="54" t="inlineStr">
+        <is>
+          <t>24/7 coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="10" t="inlineStr">
+        <is>
+          <t>Cleaner / General Labour</t>
+        </is>
+      </c>
+      <c r="B155" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="C155" s="46" t="n">
+        <v>350</v>
+      </c>
+      <c r="D155" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E155" s="22">
+        <f>B155*C155</f>
+        <v/>
+      </c>
+      <c r="F155" s="54" t="inlineStr">
+        <is>
+          <t>Site-wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="15" t="inlineStr">
+        <is>
+          <t>TOTAL STAFFING</t>
+        </is>
+      </c>
+      <c r="B156" s="55">
+        <f>SUM(B121:B155)</f>
+        <v/>
+      </c>
+      <c r="E156" s="51">
+        <f>SUM(E121:E155)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="7" t="inlineStr">
+        <is>
+          <t>ANNUAL LABOUR COST (x12 months)</t>
+        </is>
+      </c>
+      <c r="E157" s="22">
+        <f>E156*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL CAPEX SUMMARY</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="n"/>
+      <c r="C159" s="3" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="38" t="inlineStr">
+        <is>
+          <t>TOTAL CAPEX</t>
+        </is>
+      </c>
+      <c r="B160" s="51">
+        <f>IFERROR(SUM(B5:B159),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>MONTHLY OPERATING EXPENDITURE (OPEX)</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="n"/>
+      <c r="C162" s="3" t="n"/>
+      <c r="D162" s="3" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="9" t="inlineStr">
+        <is>
+          <t>Cost Item</t>
+        </is>
+      </c>
+      <c r="B163" s="9" t="inlineStr">
+        <is>
+          <t>Monthly Cost (USD)</t>
+        </is>
+      </c>
+      <c r="C163" s="9" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="10" t="inlineStr">
+        <is>
+          <t>Chemical Treatment</t>
+        </is>
+      </c>
+      <c r="B164" s="22">
+        <f>IFERROR(S2_Chemical_Treatment!B33,0)</f>
+        <v/>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>From Stage 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="10" t="inlineStr">
+        <is>
+          <t>Biological Treatment</t>
+        </is>
+      </c>
+      <c r="B165" s="22">
+        <f>IFERROR(S3_Biological_Treatment!B33,0)</f>
+        <v/>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>From Stage 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="10" t="inlineStr">
+        <is>
+          <t>BSF Neonates</t>
+        </is>
+      </c>
+      <c r="B166" s="22">
+        <f>IFERROR(S4_BSF_Rearing!B8,0)</f>
+        <v/>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>From Stage 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="10" t="inlineStr">
+        <is>
+          <t>Processing (S5B)</t>
+        </is>
+      </c>
+      <c r="B167" s="22">
+        <f>IFERROR(S5B_BSF_Extraction!B29,0)</f>
+        <v/>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>From Stage 5B</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="10" t="inlineStr">
+        <is>
+          <t>Energy / Utilities</t>
+        </is>
+      </c>
+      <c r="B168" s="22">
+        <f>IFERROR(S1_Preprocessing!B30,0)</f>
+        <v/>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>From Stage 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="10" t="inlineStr">
+        <is>
+          <t>Labour (full staffing)</t>
+        </is>
+      </c>
+      <c r="B169" s="22">
+        <f>E156</f>
+        <v/>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>67 staff — see staffing section row 156</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="10" t="inlineStr">
+        <is>
+          <t>Maintenance (2% CAPEX/month)</t>
+        </is>
+      </c>
+      <c r="B170" s="22">
+        <f>IFERROR(B160*0.02/12,0)</f>
+        <v/>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>Industry standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="10" t="inlineStr">
+        <is>
+          <t>Quality Control / Lab</t>
+        </is>
+      </c>
+      <c r="B171" s="46" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>Monthly QC testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="10" t="inlineStr">
+        <is>
           <t>Transport / Logistics</t>
         </is>
       </c>
-      <c r="B112" s="46" t="n">
+      <c r="B172" s="46" t="n">
         <v>3000</v>
       </c>
-      <c r="C112" s="2" t="inlineStr">
+      <c r="C172" s="2" t="inlineStr">
         <is>
           <t>Product distribution</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="38" t="inlineStr">
+    <row r="173">
+      <c r="A173" s="38" t="inlineStr">
         <is>
           <t>TOTAL MONTHLY OPEX</t>
         </is>
       </c>
-      <c r="B113" s="52">
-        <f>IFERROR(SUM(B104:B112),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="3" t="inlineStr">
+      <c r="B173" s="52">
+        <f>IFERROR(SUM(B164:B172),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="3" t="inlineStr">
         <is>
           <t>PAYBACK &amp; NPV ANALYSIS</t>
         </is>
       </c>
-      <c r="B115" s="3" t="n"/>
-      <c r="C115" s="3" t="n"/>
-      <c r="D115" s="3" t="n"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="4" t="inlineStr">
+      <c r="B175" s="3" t="n"/>
+      <c r="C175" s="3" t="n"/>
+      <c r="D175" s="3" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="4" t="inlineStr">
         <is>
           <t>Total CAPEX</t>
         </is>
       </c>
-      <c r="B116" s="22">
-        <f>B100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="4" t="inlineStr">
+      <c r="B176" s="22">
+        <f>B160</f>
+        <v/>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="4" t="inlineStr">
         <is>
           <t>Monthly Gross Profit</t>
         </is>
       </c>
-      <c r="B117" s="22">
-        <f>IFERROR(Summary_Dashboard!B24-B113,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="38" t="inlineStr">
+      <c r="B177" s="22">
+        <f>IFERROR(Summary_Dashboard!B24-B173,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="38" t="inlineStr">
         <is>
           <t>Payback Period (months)</t>
         </is>
       </c>
-      <c r="B118" s="42">
-        <f>IFERROR(B116/B117,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="4" t="inlineStr">
+      <c r="B178" s="42">
+        <f>IFERROR(B176/B177,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="4" t="inlineStr">
         <is>
           <t>Payback Period (years)</t>
         </is>
       </c>
-      <c r="B119" s="13">
-        <f>IFERROR(B118/12,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="4" t="inlineStr">
+      <c r="B179" s="13">
+        <f>IFERROR(B178/12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="4" t="inlineStr">
         <is>
           <t>IRR Discount Rate (user-adjustable)</t>
         </is>
       </c>
-      <c r="B121" s="53" t="n">
+      <c r="B181" s="56" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="4" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="4" t="inlineStr">
         <is>
           <t>Annual Net Cash Flow</t>
         </is>
       </c>
-      <c r="B122" s="22">
-        <f>IFERROR(B117*12,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="7" t="inlineStr">
+      <c r="B182" s="22">
+        <f>IFERROR(B177*12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="7" t="inlineStr">
         <is>
           <t>5-Year NPV (simple estimate)</t>
         </is>
       </c>
-      <c r="B123" s="30">
-        <f>IFERROR(B122/(1+B121)^1+B122/(1+B121)^2+B122/(1+B121)^3+B122/(1+B121)^4+B122/(1+B121)^5-B116,0)</f>
+      <c r="B183" s="30">
+        <f>IFERROR(B182/(1+B181)^1+B182/(1+B181)^2+B182/(1+B181)^3+B182/(1+B181)^4+B182/(1+B181)^5-B176,0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Estimate DATA GAP items: add GH-ELEC $55k, remove DATA GAP flags from fire protection
- GH-ELEC (Greenhouse SCADA/sensors/zone controls): estimated $55,000
- Fire protection items ($67k) kept as estimates, red highlight removed
- Electrical total now $282,500 (was $227,500 + $55k GH-ELEC)

https://claude.ai/code/session_01WZKNxbjsTJxtui6XGx7d89
</commit_message>
<xml_diff>
--- a/CFI_Master_Excel.xlsx
+++ b/CFI_Master_Excel.xlsx
@@ -140,7 +140,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -175,12 +175,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FF4444"/>
         <bgColor rgb="00FF4444"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFCCCC"/>
-        <bgColor rgb="00FFCCCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -254,7 +248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -356,7 +350,6 @@
     <xf numFmtId="167" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4556,7 +4549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F260"/>
+  <dimension ref="A1:F261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -6021,7 +6014,7 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>ELECTRICAL PANELS &amp; CONTROLS (10 items, $227,500 — CAPEX v4.1)</t>
+          <t>ELECTRICAL PANELS &amp; CONTROLS (11 items, $282,500 — CAPEX v4.1 + GH est.)</t>
         </is>
       </c>
       <c r="B110" s="3" t="n"/>
@@ -6195,147 +6188,147 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="7" t="inlineStr">
+      <c r="A122" s="10" t="inlineStr">
+        <is>
+          <t>GH-ELEC — Greenhouse Internal Electrical (SCADA, sensors, zone controls) est.</t>
+        </is>
+      </c>
+      <c r="B122" s="46" t="n">
+        <v>55000</v>
+      </c>
+      <c r="C122" s="10" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="7" t="inlineStr">
         <is>
           <t>Electrical Subtotal</t>
         </is>
       </c>
-      <c r="B122" s="22">
-        <f>SUM(B112:B121)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="3" t="inlineStr">
-        <is>
-          <t>FIRE PROTECTION — ADDITIONAL (NOT in A8, DATA GAP — RFQ required)</t>
-        </is>
-      </c>
-      <c r="B124" s="3" t="n"/>
-      <c r="C124" s="3" t="n"/>
+      <c r="B123" s="22">
+        <f>SUM(B112:B122)</f>
+        <v/>
+      </c>
     </row>
     <row r="125">
-      <c r="A125" s="9" t="inlineStr">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>FIRE PROTECTION — ADDITIONAL (NOT in A8, estimated)</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="n"/>
+      <c r="C125" s="3" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="9" t="inlineStr">
         <is>
           <t>Equipment / Item</t>
         </is>
       </c>
-      <c r="B125" s="9" t="inlineStr">
+      <c r="B126" s="9" t="inlineStr">
         <is>
           <t>Estimated Cost (USD)</t>
         </is>
       </c>
-      <c r="C125" s="9" t="inlineStr">
+      <c r="C126" s="9" t="inlineStr">
         <is>
           <t>Category</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="10" t="inlineStr">
-        <is>
-          <t>FIRE-HYDRANT-01 — Fire Hydrant Network (100mm mains, 16 bar) DATA GAP RFQ</t>
-        </is>
-      </c>
-      <c r="B126" s="53" t="n">
-        <v>20000</v>
-      </c>
-      <c r="C126" s="10" t="inlineStr">
-        <is>
-          <t>Fire/DATA GAP</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
         <is>
-          <t>FIRE-ALARM-01 — Fire Alarm System (detectors, panel, sirens) DATA GAP</t>
-        </is>
-      </c>
-      <c r="B127" s="53" t="n">
-        <v>12000</v>
+          <t>FIRE-HYDRANT-01 — Fire Hydrant Network (100mm mains, 16 bar) est.</t>
+        </is>
+      </c>
+      <c r="B127" s="46" t="n">
+        <v>20000</v>
       </c>
       <c r="C127" s="10" t="inlineStr">
         <is>
-          <t>Fire/DATA GAP</t>
+          <t>Fire/Est.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="10" t="inlineStr">
         <is>
-          <t>FIRE-SUPPRESS-01 — Building Fire Suppression S1 (sprinkler/CO2) DATA GAP</t>
-        </is>
-      </c>
-      <c r="B128" s="53" t="n">
+          <t>FIRE-ALARM-01 — Fire Alarm System (detectors, panel, sirens) est.</t>
+        </is>
+      </c>
+      <c r="B128" s="46" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C128" s="10" t="inlineStr">
+        <is>
+          <t>Fire/Est.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="10" t="inlineStr">
+        <is>
+          <t>FIRE-SUPPRESS-01 — Building Fire Suppression S1 (sprinkler/CO2) est.</t>
+        </is>
+      </c>
+      <c r="B129" s="46" t="n">
         <v>35000</v>
       </c>
-      <c r="C128" s="10" t="inlineStr">
-        <is>
-          <t>Fire/DATA GAP</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="7" t="inlineStr">
+      <c r="C129" s="10" t="inlineStr">
+        <is>
+          <t>Fire/Est.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="7" t="inlineStr">
         <is>
           <t>Fire Protection Additional Subtotal</t>
         </is>
       </c>
-      <c r="B129" s="22">
-        <f>SUM(B126:B128)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="3" t="inlineStr">
+      <c r="B130" s="22">
+        <f>SUM(B127:B129)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr">
         <is>
           <t>BSF GREENHOUSE + IoT + AUTOMATION (20,000 m2)</t>
         </is>
       </c>
-      <c r="B131" s="3" t="n"/>
-      <c r="C131" s="3" t="n"/>
-    </row>
-    <row r="132">
-      <c r="A132" s="9" t="inlineStr">
+      <c r="B132" s="3" t="n"/>
+      <c r="C132" s="3" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="9" t="inlineStr">
         <is>
           <t>Equipment / Item</t>
         </is>
       </c>
-      <c r="B132" s="9" t="inlineStr">
+      <c r="B133" s="9" t="inlineStr">
         <is>
           <t>Estimated Cost (USD)</t>
         </is>
       </c>
-      <c r="C132" s="9" t="inlineStr">
+      <c r="C133" s="9" t="inlineStr">
         <is>
           <t>Category</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="10" t="inlineStr">
-        <is>
-          <t>Greenhouse Structure — Steel frame, poly-carbonate panels (20,000 m2)</t>
-        </is>
-      </c>
-      <c r="B133" s="46" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="C133" s="10" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
         <is>
-          <t>Greenhouse Foundation — Concrete slab + drainage (20,000 m2)</t>
+          <t>Greenhouse Structure — Steel frame, poly-carbonate panels (20,000 m2)</t>
         </is>
       </c>
       <c r="B134" s="46" t="n">
-        <v>400000</v>
+        <v>1200000</v>
       </c>
       <c r="C134" s="10" t="inlineStr">
         <is>
@@ -6346,11 +6339,11 @@
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
         <is>
-          <t>Internal Partition Walls — BSF zone separation (40 bays x 500m2)</t>
+          <t>Greenhouse Foundation — Concrete slab + drainage (20,000 m2)</t>
         </is>
       </c>
       <c r="B135" s="46" t="n">
-        <v>120000</v>
+        <v>400000</v>
       </c>
       <c r="C135" s="10" t="inlineStr">
         <is>
@@ -6361,11 +6354,11 @@
     <row r="136">
       <c r="A136" s="10" t="inlineStr">
         <is>
-          <t>Rearing Tray System — Stacked 3-tier racks (20,000 m2 effective)</t>
+          <t>Internal Partition Walls — BSF zone separation (40 bays x 500m2)</t>
         </is>
       </c>
       <c r="B136" s="46" t="n">
-        <v>350000</v>
+        <v>120000</v>
       </c>
       <c r="C136" s="10" t="inlineStr">
         <is>
@@ -6376,11 +6369,11 @@
     <row r="137">
       <c r="A137" s="10" t="inlineStr">
         <is>
-          <t>Blackout System — UV-blocking curtains + light baffles</t>
+          <t>Rearing Tray System — Stacked 3-tier racks (20,000 m2 effective)</t>
         </is>
       </c>
       <c r="B137" s="46" t="n">
-        <v>80000</v>
+        <v>350000</v>
       </c>
       <c r="C137" s="10" t="inlineStr">
         <is>
@@ -6391,11 +6384,11 @@
     <row r="138">
       <c r="A138" s="10" t="inlineStr">
         <is>
-          <t>HVAC System — Evaporative cooling + exhaust fans (20,000 m2)</t>
+          <t>Blackout System — UV-blocking curtains + light baffles</t>
         </is>
       </c>
       <c r="B138" s="46" t="n">
-        <v>280000</v>
+        <v>80000</v>
       </c>
       <c r="C138" s="10" t="inlineStr">
         <is>
@@ -6406,11 +6399,11 @@
     <row r="139">
       <c r="A139" s="10" t="inlineStr">
         <is>
-          <t>Heating System — Hot water pipes from mill waste heat</t>
+          <t>HVAC System — Evaporative cooling + exhaust fans (20,000 m2)</t>
         </is>
       </c>
       <c r="B139" s="46" t="n">
-        <v>150000</v>
+        <v>280000</v>
       </c>
       <c r="C139" s="10" t="inlineStr">
         <is>
@@ -6421,11 +6414,11 @@
     <row r="140">
       <c r="A140" s="10" t="inlineStr">
         <is>
-          <t>Humidification System — Fogging nozzles + RH control</t>
+          <t>Heating System — Hot water pipes from mill waste heat</t>
         </is>
       </c>
       <c r="B140" s="46" t="n">
-        <v>65000</v>
+        <v>150000</v>
       </c>
       <c r="C140" s="10" t="inlineStr">
         <is>
@@ -6436,11 +6429,11 @@
     <row r="141">
       <c r="A141" s="10" t="inlineStr">
         <is>
-          <t>Air Circulation Fans — 120 units, ceiling mount</t>
+          <t>Humidification System — Fogging nozzles + RH control</t>
         </is>
       </c>
       <c r="B141" s="46" t="n">
-        <v>48000</v>
+        <v>65000</v>
       </c>
       <c r="C141" s="10" t="inlineStr">
         <is>
@@ -6451,26 +6444,26 @@
     <row r="142">
       <c r="A142" s="10" t="inlineStr">
         <is>
-          <t>IoT Temperature Sensors — 200 units (5 per bay, wireless)</t>
+          <t>Air Circulation Fans — 120 units, ceiling mount</t>
         </is>
       </c>
       <c r="B142" s="46" t="n">
-        <v>30000</v>
+        <v>48000</v>
       </c>
       <c r="C142" s="10" t="inlineStr">
         <is>
-          <t>IoT/Automation</t>
+          <t>Greenhouse</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="10" t="inlineStr">
         <is>
-          <t>IoT Humidity Sensors — 200 units (5 per bay, wireless)</t>
+          <t>IoT Temperature Sensors — 200 units (5 per bay, wireless)</t>
         </is>
       </c>
       <c r="B143" s="46" t="n">
-        <v>25000</v>
+        <v>30000</v>
       </c>
       <c r="C143" s="10" t="inlineStr">
         <is>
@@ -6481,11 +6474,11 @@
     <row r="144">
       <c r="A144" s="10" t="inlineStr">
         <is>
-          <t>IoT CO2 Sensors — 40 units (1 per bay)</t>
+          <t>IoT Humidity Sensors — 200 units (5 per bay, wireless)</t>
         </is>
       </c>
       <c r="B144" s="46" t="n">
-        <v>16000</v>
+        <v>25000</v>
       </c>
       <c r="C144" s="10" t="inlineStr">
         <is>
@@ -6496,11 +6489,11 @@
     <row r="145">
       <c r="A145" s="10" t="inlineStr">
         <is>
-          <t>IoT pH Sensors — substrate monitoring, 80 units</t>
+          <t>IoT CO2 Sensors — 40 units (1 per bay)</t>
         </is>
       </c>
       <c r="B145" s="46" t="n">
-        <v>24000</v>
+        <v>16000</v>
       </c>
       <c r="C145" s="10" t="inlineStr">
         <is>
@@ -6511,11 +6504,11 @@
     <row r="146">
       <c r="A146" s="10" t="inlineStr">
         <is>
-          <t>IoT Weight Sensors — tray scales for yield tracking, 200 units</t>
+          <t>IoT pH Sensors — substrate monitoring, 80 units</t>
         </is>
       </c>
       <c r="B146" s="46" t="n">
-        <v>40000</v>
+        <v>24000</v>
       </c>
       <c r="C146" s="10" t="inlineStr">
         <is>
@@ -6526,11 +6519,11 @@
     <row r="147">
       <c r="A147" s="10" t="inlineStr">
         <is>
-          <t>IoT Ammonia Sensors — 40 units (1 per bay)</t>
+          <t>IoT Weight Sensors — tray scales for yield tracking, 200 units</t>
         </is>
       </c>
       <c r="B147" s="46" t="n">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="C147" s="10" t="inlineStr">
         <is>
@@ -6541,11 +6534,11 @@
     <row r="148">
       <c r="A148" s="10" t="inlineStr">
         <is>
-          <t>Central IoT Gateway — LoRaWAN/WiFi hub + cloud dashboard</t>
+          <t>IoT Ammonia Sensors — 40 units (1 per bay)</t>
         </is>
       </c>
       <c r="B148" s="46" t="n">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="C148" s="10" t="inlineStr">
         <is>
@@ -6556,11 +6549,11 @@
     <row r="149">
       <c r="A149" s="10" t="inlineStr">
         <is>
-          <t>IoT Software Platform — Dashboard, alerts, analytics (annual license)</t>
+          <t>Central IoT Gateway — LoRaWAN/WiFi hub + cloud dashboard</t>
         </is>
       </c>
       <c r="B149" s="46" t="n">
-        <v>25000</v>
+        <v>15000</v>
       </c>
       <c r="C149" s="10" t="inlineStr">
         <is>
@@ -6571,26 +6564,26 @@
     <row r="150">
       <c r="A150" s="10" t="inlineStr">
         <is>
-          <t>Automated Feed Distribution System — conveyor + metering</t>
+          <t>IoT Software Platform — Dashboard, alerts, analytics (annual license)</t>
         </is>
       </c>
       <c r="B150" s="46" t="n">
-        <v>180000</v>
+        <v>25000</v>
       </c>
       <c r="C150" s="10" t="inlineStr">
         <is>
-          <t>Automation</t>
+          <t>IoT/Automation</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="10" t="inlineStr">
         <is>
-          <t>Automated Larvae Harvesting System — vibrating separator + conveyor</t>
+          <t>Automated Feed Distribution System — conveyor + metering</t>
         </is>
       </c>
       <c r="B151" s="46" t="n">
-        <v>220000</v>
+        <v>180000</v>
       </c>
       <c r="C151" s="10" t="inlineStr">
         <is>
@@ -6601,11 +6594,11 @@
     <row r="152">
       <c r="A152" s="10" t="inlineStr">
         <is>
-          <t>Automated Tray Washing Station</t>
+          <t>Automated Larvae Harvesting System — vibrating separator + conveyor</t>
         </is>
       </c>
       <c r="B152" s="46" t="n">
-        <v>45000</v>
+        <v>220000</v>
       </c>
       <c r="C152" s="10" t="inlineStr">
         <is>
@@ -6616,26 +6609,26 @@
     <row r="153">
       <c r="A153" s="10" t="inlineStr">
         <is>
-          <t>Automated Climate Control PLC — Siemens/Allen-Bradley</t>
+          <t>Automated Tray Washing Station</t>
         </is>
       </c>
       <c r="B153" s="46" t="n">
-        <v>35000</v>
+        <v>45000</v>
       </c>
       <c r="C153" s="10" t="inlineStr">
         <is>
-          <t>IoT/Automation</t>
+          <t>Automation</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="10" t="inlineStr">
         <is>
-          <t>SCADA System — Central control room, 4 screens</t>
+          <t>Automated Climate Control PLC — Siemens/Allen-Bradley</t>
         </is>
       </c>
       <c r="B154" s="46" t="n">
-        <v>40000</v>
+        <v>35000</v>
       </c>
       <c r="C154" s="10" t="inlineStr">
         <is>
@@ -6646,26 +6639,26 @@
     <row r="155">
       <c r="A155" s="10" t="inlineStr">
         <is>
-          <t>Water Supply System — treatment + distribution (20,000 m2)</t>
+          <t>SCADA System — Central control room, 4 screens</t>
         </is>
       </c>
       <c r="B155" s="46" t="n">
-        <v>85000</v>
+        <v>40000</v>
       </c>
       <c r="C155" s="10" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>IoT/Automation</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="10" t="inlineStr">
         <is>
-          <t>Electrical Distribution — panels, cabling, backup genset</t>
+          <t>Water Supply System — treatment + distribution (20,000 m2)</t>
         </is>
       </c>
       <c r="B156" s="46" t="n">
-        <v>120000</v>
+        <v>85000</v>
       </c>
       <c r="C156" s="10" t="inlineStr">
         <is>
@@ -6676,11 +6669,11 @@
     <row r="157">
       <c r="A157" s="10" t="inlineStr">
         <is>
-          <t>Waste Water Treatment — effluent from rearing</t>
+          <t>Electrical Distribution — panels, cabling, backup genset</t>
         </is>
       </c>
       <c r="B157" s="46" t="n">
-        <v>60000</v>
+        <v>120000</v>
       </c>
       <c r="C157" s="10" t="inlineStr">
         <is>
@@ -6691,41 +6684,41 @@
     <row r="158">
       <c r="A158" s="10" t="inlineStr">
         <is>
-          <t>Fire Suppression System</t>
+          <t>Waste Water Treatment — effluent from rearing</t>
         </is>
       </c>
       <c r="B158" s="46" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="C158" s="10" t="inlineStr">
         <is>
-          <t>Facilities</t>
+          <t>Utilities</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="10" t="inlineStr">
         <is>
-          <t>Site Clearing &amp; Grading (2.5 ha total footprint)</t>
+          <t>Fire Suppression System</t>
         </is>
       </c>
       <c r="B159" s="46" t="n">
-        <v>80000</v>
+        <v>45000</v>
       </c>
       <c r="C159" s="10" t="inlineStr">
         <is>
-          <t>Site Works</t>
+          <t>Facilities</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="10" t="inlineStr">
         <is>
-          <t>Access Roads — Internal + connection to mill (500m gravel)</t>
+          <t>Site Clearing &amp; Grading (2.5 ha total footprint)</t>
         </is>
       </c>
       <c r="B160" s="46" t="n">
-        <v>60000</v>
+        <v>80000</v>
       </c>
       <c r="C160" s="10" t="inlineStr">
         <is>
@@ -6736,41 +6729,41 @@
     <row r="161">
       <c r="A161" s="10" t="inlineStr">
         <is>
-          <t>Perimeter Fencing + Security</t>
+          <t>Access Roads — Internal + connection to mill (500m gravel)</t>
         </is>
       </c>
       <c r="B161" s="46" t="n">
-        <v>35000</v>
+        <v>60000</v>
       </c>
       <c r="C161" s="10" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>Site Works</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="10" t="inlineStr">
         <is>
-          <t>Drainage System — Surface + subsurface</t>
+          <t>Perimeter Fencing + Security</t>
         </is>
       </c>
       <c r="B162" s="46" t="n">
-        <v>55000</v>
+        <v>35000</v>
       </c>
       <c r="C162" s="10" t="inlineStr">
         <is>
-          <t>Site Works</t>
+          <t>Greenhouse</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="10" t="inlineStr">
         <is>
-          <t>Landscaping + Erosion Control</t>
+          <t>Drainage System — Surface + subsurface</t>
         </is>
       </c>
       <c r="B163" s="46" t="n">
-        <v>20000</v>
+        <v>55000</v>
       </c>
       <c r="C163" s="10" t="inlineStr">
         <is>
@@ -6781,76 +6774,76 @@
     <row r="164">
       <c r="A164" s="10" t="inlineStr">
         <is>
-          <t>Staff Facilities — Office, changing rooms, canteen</t>
+          <t>Landscaping + Erosion Control</t>
         </is>
       </c>
       <c r="B164" s="46" t="n">
-        <v>85000</v>
+        <v>20000</v>
       </c>
       <c r="C164" s="10" t="inlineStr">
         <is>
-          <t>Facilities</t>
+          <t>Site Works</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="10" t="inlineStr">
         <is>
+          <t>Staff Facilities — Office, changing rooms, canteen</t>
+        </is>
+      </c>
+      <c r="B165" s="46" t="n">
+        <v>85000</v>
+      </c>
+      <c r="C165" s="10" t="inlineStr">
+        <is>
+          <t>Facilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="10" t="inlineStr">
+        <is>
           <t>Storage Warehouse — Finished product (500 m2)</t>
         </is>
       </c>
-      <c r="B165" s="46" t="n">
+      <c r="B166" s="46" t="n">
         <v>120000</v>
       </c>
-      <c r="C165" s="10" t="inlineStr">
+      <c r="C166" s="10" t="inlineStr">
         <is>
           <t>Facilities</t>
         </is>
       </c>
     </row>
-    <row r="166">
-      <c r="A166" s="7" t="inlineStr">
+    <row r="167">
+      <c r="A167" s="7" t="inlineStr">
         <is>
           <t>Greenhouse + IoT Subtotal</t>
         </is>
       </c>
-      <c r="B166" s="22">
-        <f>SUM(B133:B165)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="3" t="inlineStr">
+      <c r="B167" s="22">
+        <f>SUM(B134:B166)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="3" t="inlineStr">
         <is>
           <t>S5 EXTRACTION &amp; POST-PROCESSING</t>
         </is>
       </c>
-      <c r="B168" s="3" t="n"/>
-      <c r="C168" s="3" t="n"/>
-    </row>
-    <row r="169">
-      <c r="A169" s="10" t="inlineStr">
-        <is>
-          <t>S5A — Frass screening/bagging line</t>
-        </is>
-      </c>
-      <c r="B169" s="46" t="n">
-        <v>20000</v>
-      </c>
-      <c r="C169" s="10" t="inlineStr">
-        <is>
-          <t>S5/Lab</t>
-        </is>
-      </c>
+      <c r="B169" s="3" t="n"/>
+      <c r="C169" s="3" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="10" t="inlineStr">
         <is>
-          <t>S5B — Larvae separation (vibrating + thermal)</t>
+          <t>S5A — Frass screening/bagging line</t>
         </is>
       </c>
       <c r="B170" s="46" t="n">
-        <v>30000</v>
+        <v>20000</v>
       </c>
       <c r="C170" s="10" t="inlineStr">
         <is>
@@ -6861,11 +6854,11 @@
     <row r="171">
       <c r="A171" s="10" t="inlineStr">
         <is>
-          <t>S5B — Oil press (screw type, 85% eff)</t>
+          <t>S5B — Larvae separation (vibrating + thermal)</t>
         </is>
       </c>
       <c r="B171" s="46" t="n">
-        <v>45000</v>
+        <v>30000</v>
       </c>
       <c r="C171" s="10" t="inlineStr">
         <is>
@@ -6876,11 +6869,11 @@
     <row r="172">
       <c r="A172" s="10" t="inlineStr">
         <is>
-          <t>S5B — Drying system (belt dryer)</t>
+          <t>S5B — Oil press (screw type, 85% eff)</t>
         </is>
       </c>
       <c r="B172" s="46" t="n">
-        <v>40000</v>
+        <v>45000</v>
       </c>
       <c r="C172" s="10" t="inlineStr">
         <is>
@@ -6891,78 +6884,78 @@
     <row r="173">
       <c r="A173" s="10" t="inlineStr">
         <is>
+          <t>S5B — Drying system (belt dryer)</t>
+        </is>
+      </c>
+      <c r="B173" s="46" t="n">
+        <v>40000</v>
+      </c>
+      <c r="C173" s="10" t="inlineStr">
+        <is>
+          <t>S5/Lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="10" t="inlineStr">
+        <is>
           <t>Laboratory — QC lab (ICP-OES capable)</t>
         </is>
       </c>
-      <c r="B173" s="46" t="n">
+      <c r="B174" s="46" t="n">
         <v>45000</v>
       </c>
-      <c r="C173" s="10" t="inlineStr">
+      <c r="C174" s="10" t="inlineStr">
         <is>
           <t>S5/Lab</t>
         </is>
       </c>
     </row>
-    <row r="174">
-      <c r="A174" s="7" t="inlineStr">
+    <row r="175">
+      <c r="A175" s="7" t="inlineStr">
         <is>
           <t>S5 Subtotal</t>
         </is>
       </c>
-      <c r="B174" s="22">
-        <f>SUM(B169:B173)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="3" t="inlineStr">
+      <c r="B175" s="22">
+        <f>SUM(B170:B174)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="3" t="inlineStr">
         <is>
           <t>MOBILE EQUIPMENT &amp; VEHICLES</t>
         </is>
       </c>
-      <c r="B176" s="3" t="n"/>
-      <c r="C176" s="3" t="n"/>
-    </row>
-    <row r="177">
-      <c r="A177" s="9" t="inlineStr">
+      <c r="B177" s="3" t="n"/>
+      <c r="C177" s="3" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="9" t="inlineStr">
         <is>
           <t>Equipment / Item</t>
         </is>
       </c>
-      <c r="B177" s="9" t="inlineStr">
+      <c r="B178" s="9" t="inlineStr">
         <is>
           <t>Estimated Cost (USD)</t>
         </is>
       </c>
-      <c r="C177" s="9" t="inlineStr">
+      <c r="C178" s="9" t="inlineStr">
         <is>
           <t>Category</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="10" t="inlineStr">
-        <is>
-          <t>Wheel Loader — Komatsu WA100 or equiv (1.0m3 bucket, EFB/OPDC handling)</t>
-        </is>
-      </c>
-      <c r="B178" s="46" t="n">
-        <v>85000</v>
-      </c>
-      <c r="C178" s="10" t="inlineStr">
-        <is>
-          <t>Mobile</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="10" t="inlineStr">
         <is>
-          <t>Wheel Loader — Komatsu WA70 or equiv (0.5m3 bucket, PKSA/compost)</t>
+          <t>Wheel Loader — Komatsu WA100 or equiv (1.0m3 bucket, EFB/OPDC handling)</t>
         </is>
       </c>
       <c r="B179" s="46" t="n">
-        <v>55000</v>
+        <v>85000</v>
       </c>
       <c r="C179" s="10" t="inlineStr">
         <is>
@@ -6973,11 +6966,11 @@
     <row r="180">
       <c r="A180" s="10" t="inlineStr">
         <is>
-          <t>Skid-Steer Loader / Bobcat — S650 or equiv (BSF frass, substrate)</t>
+          <t>Wheel Loader — Komatsu WA70 or equiv (0.5m3 bucket, PKSA/compost)</t>
         </is>
       </c>
       <c r="B180" s="46" t="n">
-        <v>45000</v>
+        <v>55000</v>
       </c>
       <c r="C180" s="10" t="inlineStr">
         <is>
@@ -6988,11 +6981,11 @@
     <row r="181">
       <c r="A181" s="10" t="inlineStr">
         <is>
-          <t>Skid-Steer Loader / Bobcat — S450 or equiv (greenhouse internal)</t>
+          <t>Skid-Steer Loader / Bobcat — S650 or equiv (BSF frass, substrate)</t>
         </is>
       </c>
       <c r="B181" s="46" t="n">
-        <v>38000</v>
+        <v>45000</v>
       </c>
       <c r="C181" s="10" t="inlineStr">
         <is>
@@ -7003,11 +6996,11 @@
     <row r="182">
       <c r="A182" s="10" t="inlineStr">
         <is>
-          <t>Mini Excavator — 3.5t (site maintenance, drainage, pit cleaning)</t>
+          <t>Skid-Steer Loader / Bobcat — S450 or equiv (greenhouse internal)</t>
         </is>
       </c>
       <c r="B182" s="46" t="n">
-        <v>42000</v>
+        <v>38000</v>
       </c>
       <c r="C182" s="10" t="inlineStr">
         <is>
@@ -7018,11 +7011,11 @@
     <row r="183">
       <c r="A183" s="10" t="inlineStr">
         <is>
-          <t>Dump Truck — 10t (EFB transport mill to S1, internal)</t>
+          <t>Mini Excavator — 3.5t (site maintenance, drainage, pit cleaning)</t>
         </is>
       </c>
       <c r="B183" s="46" t="n">
-        <v>65000</v>
+        <v>42000</v>
       </c>
       <c r="C183" s="10" t="inlineStr">
         <is>
@@ -7033,7 +7026,7 @@
     <row r="184">
       <c r="A184" s="10" t="inlineStr">
         <is>
-          <t>Dump Truck — 10t (OPDC/POS transport mill to S1)</t>
+          <t>Dump Truck — 10t (EFB transport mill to S1, internal)</t>
         </is>
       </c>
       <c r="B184" s="46" t="n">
@@ -7048,11 +7041,11 @@
     <row r="185">
       <c r="A185" s="10" t="inlineStr">
         <is>
-          <t>Flatbed Truck — 8t (finished product transport, frass/meal)</t>
+          <t>Dump Truck — 10t (OPDC/POS transport mill to S1)</t>
         </is>
       </c>
       <c r="B185" s="46" t="n">
-        <v>55000</v>
+        <v>65000</v>
       </c>
       <c r="C185" s="10" t="inlineStr">
         <is>
@@ -7063,11 +7056,11 @@
     <row r="186">
       <c r="A186" s="10" t="inlineStr">
         <is>
-          <t>Tanker Truck — 5,000L (water, POME, liquid transfer)</t>
+          <t>Flatbed Truck — 8t (finished product transport, frass/meal)</t>
         </is>
       </c>
       <c r="B186" s="46" t="n">
-        <v>48000</v>
+        <v>55000</v>
       </c>
       <c r="C186" s="10" t="inlineStr">
         <is>
@@ -7078,11 +7071,11 @@
     <row r="187">
       <c r="A187" s="10" t="inlineStr">
         <is>
-          <t>Pickup Truck — 4x4 (site management, 2 units)</t>
+          <t>Tanker Truck — 5,000L (water, POME, liquid transfer)</t>
         </is>
       </c>
       <c r="B187" s="46" t="n">
-        <v>60000</v>
+        <v>48000</v>
       </c>
       <c r="C187" s="10" t="inlineStr">
         <is>
@@ -7093,11 +7086,11 @@
     <row r="188">
       <c r="A188" s="10" t="inlineStr">
         <is>
-          <t>Forklift — 3t diesel (warehouse, bagged product, 2 units)</t>
+          <t>Pickup Truck — 4x4 (site management, 2 units)</t>
         </is>
       </c>
       <c r="B188" s="46" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="C188" s="10" t="inlineStr">
         <is>
@@ -7108,11 +7101,11 @@
     <row r="189">
       <c r="A189" s="10" t="inlineStr">
         <is>
-          <t>Forklift — 1.5t electric (greenhouse internal, 2 units)</t>
+          <t>Forklift — 3t diesel (warehouse, bagged product, 2 units)</t>
         </is>
       </c>
       <c r="B189" s="46" t="n">
-        <v>36000</v>
+        <v>50000</v>
       </c>
       <c r="C189" s="10" t="inlineStr">
         <is>
@@ -7123,11 +7116,11 @@
     <row r="190">
       <c r="A190" s="10" t="inlineStr">
         <is>
-          <t>Tipping Trailer — 8t (substrate/frass haulage, 2 units)</t>
+          <t>Forklift — 1.5t electric (greenhouse internal, 2 units)</t>
         </is>
       </c>
       <c r="B190" s="46" t="n">
-        <v>24000</v>
+        <v>36000</v>
       </c>
       <c r="C190" s="10" t="inlineStr">
         <is>
@@ -7138,11 +7131,11 @@
     <row r="191">
       <c r="A191" s="10" t="inlineStr">
         <is>
-          <t>Pallet Jacks — manual (4 units, warehouse)</t>
+          <t>Tipping Trailer — 8t (substrate/frass haulage, 2 units)</t>
         </is>
       </c>
       <c r="B191" s="46" t="n">
-        <v>3200</v>
+        <v>24000</v>
       </c>
       <c r="C191" s="10" t="inlineStr">
         <is>
@@ -7153,11 +7146,11 @@
     <row r="192">
       <c r="A192" s="10" t="inlineStr">
         <is>
-          <t>Grab Bucket Attachment — for wheel loader (EFB)</t>
+          <t>Pallet Jacks — manual (4 units, warehouse)</t>
         </is>
       </c>
       <c r="B192" s="46" t="n">
-        <v>8000</v>
+        <v>3200</v>
       </c>
       <c r="C192" s="10" t="inlineStr">
         <is>
@@ -7168,113 +7161,101 @@
     <row r="193">
       <c r="A193" s="10" t="inlineStr">
         <is>
+          <t>Grab Bucket Attachment — for wheel loader (EFB)</t>
+        </is>
+      </c>
+      <c r="B193" s="46" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C193" s="10" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="10" t="inlineStr">
+        <is>
           <t>Sweeper Attachment — for bobcat (greenhouse cleaning)</t>
         </is>
       </c>
-      <c r="B193" s="46" t="n">
+      <c r="B194" s="46" t="n">
         <v>6500</v>
       </c>
-      <c r="C193" s="10" t="inlineStr">
+      <c r="C194" s="10" t="inlineStr">
         <is>
           <t>Mobile</t>
         </is>
       </c>
     </row>
-    <row r="194">
-      <c r="A194" s="7" t="inlineStr">
+    <row r="195">
+      <c r="A195" s="7" t="inlineStr">
         <is>
           <t>Mobile Equipment Subtotal</t>
         </is>
       </c>
-      <c r="B194" s="22">
-        <f>SUM(B178:B193)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" s="3" t="inlineStr">
+      <c r="B195" s="22">
+        <f>SUM(B179:B194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="3" t="inlineStr">
         <is>
           <t>STAFFING — FULL HEADCOUNT &amp; LABOUR COST</t>
         </is>
       </c>
-      <c r="B196" s="3" t="n"/>
-      <c r="C196" s="3" t="n"/>
-      <c r="D196" s="3" t="n"/>
-      <c r="E196" s="3" t="n"/>
-      <c r="F196" s="3" t="n"/>
-    </row>
-    <row r="197">
-      <c r="A197" s="9" t="inlineStr">
+      <c r="B197" s="3" t="n"/>
+      <c r="C197" s="3" t="n"/>
+      <c r="D197" s="3" t="n"/>
+      <c r="E197" s="3" t="n"/>
+      <c r="F197" s="3" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="9" t="inlineStr">
         <is>
           <t>Position</t>
         </is>
       </c>
-      <c r="B197" s="9" t="inlineStr">
+      <c r="B198" s="9" t="inlineStr">
         <is>
           <t>Headcount</t>
         </is>
       </c>
-      <c r="C197" s="9" t="inlineStr">
+      <c r="C198" s="9" t="inlineStr">
         <is>
           <t>Salary (USD/month)</t>
         </is>
       </c>
-      <c r="D197" s="9" t="inlineStr">
+      <c r="D198" s="9" t="inlineStr">
         <is>
           <t>Shift</t>
         </is>
       </c>
-      <c r="E197" s="9" t="inlineStr">
+      <c r="E198" s="9" t="inlineStr">
         <is>
           <t>Monthly Cost (USD)</t>
         </is>
       </c>
-      <c r="F197" s="9" t="inlineStr">
+      <c r="F198" s="9" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" s="10" t="inlineStr">
-        <is>
-          <t>S1 — EFB Line Operator (shredder + hammer mill)</t>
-        </is>
-      </c>
-      <c r="B198" s="54" t="n">
-        <v>2</v>
-      </c>
-      <c r="C198" s="46" t="n">
-        <v>450</v>
-      </c>
-      <c r="D198" s="54" t="inlineStr">
-        <is>
-          <t>2-shift</t>
-        </is>
-      </c>
-      <c r="E198" s="22">
-        <f>B198*C198</f>
-        <v/>
-      </c>
-      <c r="F198" s="55" t="inlineStr">
-        <is>
-          <t>1 per shift, monitors feed + oversize return</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="10" t="inlineStr">
         <is>
-          <t>S1 — EFB Conveyor / Screen Operator</t>
-        </is>
-      </c>
-      <c r="B199" s="54" t="n">
+          <t>S1 — EFB Line Operator (shredder + hammer mill)</t>
+        </is>
+      </c>
+      <c r="B199" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C199" s="46" t="n">
-        <v>400</v>
-      </c>
-      <c r="D199" s="54" t="inlineStr">
+        <v>450</v>
+      </c>
+      <c r="D199" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7283,25 +7264,25 @@
         <f>B199*C199</f>
         <v/>
       </c>
-      <c r="F199" s="55" t="inlineStr">
-        <is>
-          <t>Belt + vibrating screen monitoring</t>
+      <c r="F199" s="54" t="inlineStr">
+        <is>
+          <t>1 per shift, monitors feed + oversize return</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="10" t="inlineStr">
         <is>
-          <t>S1 — EFB Screw Press Operator</t>
-        </is>
-      </c>
-      <c r="B200" s="54" t="n">
+          <t>S1 — EFB Conveyor / Screen Operator</t>
+        </is>
+      </c>
+      <c r="B200" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C200" s="46" t="n">
-        <v>450</v>
-      </c>
-      <c r="D200" s="54" t="inlineStr">
+        <v>400</v>
+      </c>
+      <c r="D200" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7310,25 +7291,25 @@
         <f>B200*C200</f>
         <v/>
       </c>
-      <c r="F200" s="55" t="inlineStr">
-        <is>
-          <t>MC control, filtrate routing</t>
+      <c r="F200" s="54" t="inlineStr">
+        <is>
+          <t>Belt + vibrating screen monitoring</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="10" t="inlineStr">
         <is>
-          <t>S1 — OPDC Line Operator (shredder + hammer mill)</t>
-        </is>
-      </c>
-      <c r="B201" s="54" t="n">
+          <t>S1 — EFB Screw Press Operator</t>
+        </is>
+      </c>
+      <c r="B201" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C201" s="46" t="n">
         <v>450</v>
       </c>
-      <c r="D201" s="54" t="inlineStr">
+      <c r="D201" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7337,21 +7318,25 @@
         <f>B201*C201</f>
         <v/>
       </c>
-      <c r="F201" s="55" t="inlineStr"/>
+      <c r="F201" s="54" t="inlineStr">
+        <is>
+          <t>MC control, filtrate routing</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="10" t="inlineStr">
         <is>
-          <t>S1 — OPDC Conveyor / Press Operator</t>
-        </is>
-      </c>
-      <c r="B202" s="54" t="n">
+          <t>S1 — OPDC Line Operator (shredder + hammer mill)</t>
+        </is>
+      </c>
+      <c r="B202" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C202" s="46" t="n">
-        <v>400</v>
-      </c>
-      <c r="D202" s="54" t="inlineStr">
+        <v>450</v>
+      </c>
+      <c r="D202" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7360,75 +7345,71 @@
         <f>B202*C202</f>
         <v/>
       </c>
-      <c r="F202" s="55" t="inlineStr"/>
+      <c r="F202" s="54" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="10" t="inlineStr">
         <is>
-          <t>S1 — POS Decanter Operator</t>
-        </is>
-      </c>
-      <c r="B203" s="54" t="n">
-        <v>1</v>
+          <t>S1 — OPDC Conveyor / Press Operator</t>
+        </is>
+      </c>
+      <c r="B203" s="53" t="n">
+        <v>2</v>
       </c>
       <c r="C203" s="46" t="n">
-        <v>550</v>
-      </c>
-      <c r="D203" s="54" t="inlineStr">
-        <is>
-          <t>day</t>
+        <v>400</v>
+      </c>
+      <c r="D203" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
         </is>
       </c>
       <c r="E203" s="22">
         <f>B203*C203</f>
         <v/>
       </c>
-      <c r="F203" s="55" t="inlineStr">
-        <is>
-          <t>Skilled: centrifuge operation + Fe gate sampling</t>
-        </is>
-      </c>
+      <c r="F203" s="54" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="10" t="inlineStr">
         <is>
-          <t>S1 — Wheel Loader Operator (EFB/OPDC feed)</t>
-        </is>
-      </c>
-      <c r="B204" s="54" t="n">
-        <v>2</v>
+          <t>S1 — POS Decanter Operator</t>
+        </is>
+      </c>
+      <c r="B204" s="53" t="n">
+        <v>1</v>
       </c>
       <c r="C204" s="46" t="n">
-        <v>500</v>
-      </c>
-      <c r="D204" s="54" t="inlineStr">
-        <is>
-          <t>2-shift</t>
+        <v>550</v>
+      </c>
+      <c r="D204" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
         </is>
       </c>
       <c r="E204" s="22">
         <f>B204*C204</f>
         <v/>
       </c>
-      <c r="F204" s="55" t="inlineStr">
-        <is>
-          <t>Komatsu WA100</t>
+      <c r="F204" s="54" t="inlineStr">
+        <is>
+          <t>Skilled: centrifuge operation + Fe gate sampling</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="10" t="inlineStr">
         <is>
-          <t>S1 — Dump Truck Driver (mill to S1)</t>
-        </is>
-      </c>
-      <c r="B205" s="54" t="n">
+          <t>S1 — Wheel Loader Operator (EFB/OPDC feed)</t>
+        </is>
+      </c>
+      <c r="B205" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C205" s="46" t="n">
-        <v>450</v>
-      </c>
-      <c r="D205" s="54" t="inlineStr">
+        <v>500</v>
+      </c>
+      <c r="D205" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7437,25 +7418,25 @@
         <f>B205*C205</f>
         <v/>
       </c>
-      <c r="F205" s="55" t="inlineStr">
-        <is>
-          <t>2x 10t dump trucks</t>
+      <c r="F205" s="54" t="inlineStr">
+        <is>
+          <t>Komatsu WA100</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="10" t="inlineStr">
         <is>
-          <t>S2 — Chemical Dosing Operator</t>
-        </is>
-      </c>
-      <c r="B206" s="54" t="n">
+          <t>S1 — Dump Truck Driver (mill to S1)</t>
+        </is>
+      </c>
+      <c r="B206" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C206" s="46" t="n">
-        <v>500</v>
-      </c>
-      <c r="D206" s="54" t="inlineStr">
+        <v>450</v>
+      </c>
+      <c r="D206" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7464,25 +7445,25 @@
         <f>B206*C206</f>
         <v/>
       </c>
-      <c r="F206" s="55" t="inlineStr">
-        <is>
-          <t>PKSA/chemical mixing, pH monitoring</t>
+      <c r="F206" s="54" t="inlineStr">
+        <is>
+          <t>2x 10t dump trucks</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="10" t="inlineStr">
         <is>
-          <t>S2 — Neutralisation Bay Attendant</t>
-        </is>
-      </c>
-      <c r="B207" s="54" t="n">
+          <t>S2 — Chemical Dosing Operator</t>
+        </is>
+      </c>
+      <c r="B207" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C207" s="46" t="n">
-        <v>400</v>
-      </c>
-      <c r="D207" s="54" t="inlineStr">
+        <v>500</v>
+      </c>
+      <c r="D207" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7491,106 +7472,106 @@
         <f>B207*C207</f>
         <v/>
       </c>
-      <c r="F207" s="55" t="inlineStr">
-        <is>
-          <t>Turnings at 8-12hr and 16-20hr</t>
+      <c r="F207" s="54" t="inlineStr">
+        <is>
+          <t>PKSA/chemical mixing, pH monitoring</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="10" t="inlineStr">
         <is>
-          <t>S3 — Biological Inoculation Technician</t>
-        </is>
-      </c>
-      <c r="B208" s="54" t="n">
-        <v>1</v>
+          <t>S2 — Neutralisation Bay Attendant</t>
+        </is>
+      </c>
+      <c r="B208" s="53" t="n">
+        <v>2</v>
       </c>
       <c r="C208" s="46" t="n">
-        <v>600</v>
-      </c>
-      <c r="D208" s="54" t="inlineStr">
-        <is>
-          <t>day</t>
+        <v>400</v>
+      </c>
+      <c r="D208" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
         </is>
       </c>
       <c r="E208" s="22">
         <f>B208*C208</f>
         <v/>
       </c>
-      <c r="F208" s="55" t="inlineStr">
-        <is>
-          <t>Consortium preparation, spray application</t>
+      <c r="F208" s="54" t="inlineStr">
+        <is>
+          <t>Turnings at 8-12hr and 16-20hr</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="10" t="inlineStr">
         <is>
-          <t>S3 — Composting / Windrow Operator</t>
-        </is>
-      </c>
-      <c r="B209" s="54" t="n">
-        <v>2</v>
+          <t>S3 — Biological Inoculation Technician</t>
+        </is>
+      </c>
+      <c r="B209" s="53" t="n">
+        <v>1</v>
       </c>
       <c r="C209" s="46" t="n">
-        <v>450</v>
-      </c>
-      <c r="D209" s="54" t="inlineStr">
-        <is>
-          <t>2-shift</t>
+        <v>600</v>
+      </c>
+      <c r="D209" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
         </is>
       </c>
       <c r="E209" s="22">
         <f>B209*C209</f>
         <v/>
       </c>
-      <c r="F209" s="55" t="inlineStr">
-        <is>
-          <t>Windrow turner + aeration monitoring</t>
+      <c r="F209" s="54" t="inlineStr">
+        <is>
+          <t>Consortium preparation, spray application</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="10" t="inlineStr">
         <is>
-          <t>S3 — Bobcat Operator (substrate handling)</t>
-        </is>
-      </c>
-      <c r="B210" s="54" t="n">
-        <v>1</v>
+          <t>S3 — Composting / Windrow Operator</t>
+        </is>
+      </c>
+      <c r="B210" s="53" t="n">
+        <v>2</v>
       </c>
       <c r="C210" s="46" t="n">
         <v>450</v>
       </c>
-      <c r="D210" s="54" t="inlineStr">
-        <is>
-          <t>day</t>
+      <c r="D210" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
         </is>
       </c>
       <c r="E210" s="22">
         <f>B210*C210</f>
         <v/>
       </c>
-      <c r="F210" s="55" t="inlineStr">
-        <is>
-          <t>S650 skid-steer</t>
+      <c r="F210" s="54" t="inlineStr">
+        <is>
+          <t>Windrow turner + aeration monitoring</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="10" t="inlineStr">
         <is>
-          <t>S4 — Greenhouse Supervisor</t>
-        </is>
-      </c>
-      <c r="B211" s="54" t="n">
+          <t>S3 — Bobcat Operator (substrate handling)</t>
+        </is>
+      </c>
+      <c r="B211" s="53" t="n">
         <v>1</v>
       </c>
       <c r="C211" s="46" t="n">
-        <v>900</v>
-      </c>
-      <c r="D211" s="54" t="inlineStr">
+        <v>450</v>
+      </c>
+      <c r="D211" s="53" t="inlineStr">
         <is>
           <t>day</t>
         </is>
@@ -7599,52 +7580,52 @@
         <f>B211*C211</f>
         <v/>
       </c>
-      <c r="F211" s="55" t="inlineStr">
-        <is>
-          <t>Overall BSF rearing management</t>
+      <c r="F211" s="54" t="inlineStr">
+        <is>
+          <t>S650 skid-steer</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="10" t="inlineStr">
         <is>
-          <t>S4 — BSF Tray Attendant (feeding + monitoring)</t>
-        </is>
-      </c>
-      <c r="B212" s="54" t="n">
-        <v>8</v>
+          <t>S4 — Greenhouse Supervisor</t>
+        </is>
+      </c>
+      <c r="B212" s="53" t="n">
+        <v>1</v>
       </c>
       <c r="C212" s="46" t="n">
-        <v>400</v>
-      </c>
-      <c r="D212" s="54" t="inlineStr">
-        <is>
-          <t>2-shift</t>
+        <v>900</v>
+      </c>
+      <c r="D212" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
         </is>
       </c>
       <c r="E212" s="22">
         <f>B212*C212</f>
         <v/>
       </c>
-      <c r="F212" s="55" t="inlineStr">
-        <is>
-          <t>4 per shift, 5000m2 per attendant</t>
+      <c r="F212" s="54" t="inlineStr">
+        <is>
+          <t>Overall BSF rearing management</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="10" t="inlineStr">
         <is>
-          <t>S4 — BSF Neonate Nursery Technician</t>
-        </is>
-      </c>
-      <c r="B213" s="54" t="n">
-        <v>2</v>
+          <t>S4 — BSF Tray Attendant (feeding + monitoring)</t>
+        </is>
+      </c>
+      <c r="B213" s="53" t="n">
+        <v>8</v>
       </c>
       <c r="C213" s="46" t="n">
-        <v>550</v>
-      </c>
-      <c r="D213" s="54" t="inlineStr">
+        <v>400</v>
+      </c>
+      <c r="D213" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7653,79 +7634,79 @@
         <f>B213*C213</f>
         <v/>
       </c>
-      <c r="F213" s="55" t="inlineStr">
-        <is>
-          <t>Colony management, egg collection</t>
+      <c r="F213" s="54" t="inlineStr">
+        <is>
+          <t>4 per shift, 5000m2 per attendant</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="10" t="inlineStr">
         <is>
-          <t>S4 — Greenhouse Climate / IoT Technician</t>
-        </is>
-      </c>
-      <c r="B214" s="54" t="n">
-        <v>1</v>
+          <t>S4 — BSF Neonate Nursery Technician</t>
+        </is>
+      </c>
+      <c r="B214" s="53" t="n">
+        <v>2</v>
       </c>
       <c r="C214" s="46" t="n">
-        <v>700</v>
-      </c>
-      <c r="D214" s="54" t="inlineStr">
-        <is>
-          <t>day</t>
+        <v>550</v>
+      </c>
+      <c r="D214" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
         </is>
       </c>
       <c r="E214" s="22">
         <f>B214*C214</f>
         <v/>
       </c>
-      <c r="F214" s="55" t="inlineStr">
-        <is>
-          <t>SCADA/PLC, sensor maintenance</t>
+      <c r="F214" s="54" t="inlineStr">
+        <is>
+          <t>Colony management, egg collection</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="10" t="inlineStr">
         <is>
-          <t>S4 — Bobcat Operator (greenhouse internal)</t>
-        </is>
-      </c>
-      <c r="B215" s="54" t="n">
-        <v>2</v>
+          <t>S4 — Greenhouse Climate / IoT Technician</t>
+        </is>
+      </c>
+      <c r="B215" s="53" t="n">
+        <v>1</v>
       </c>
       <c r="C215" s="46" t="n">
-        <v>450</v>
-      </c>
-      <c r="D215" s="54" t="inlineStr">
-        <is>
-          <t>2-shift</t>
+        <v>700</v>
+      </c>
+      <c r="D215" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
         </is>
       </c>
       <c r="E215" s="22">
         <f>B215*C215</f>
         <v/>
       </c>
-      <c r="F215" s="55" t="inlineStr">
-        <is>
-          <t>S450, substrate + frass movement</t>
+      <c r="F215" s="54" t="inlineStr">
+        <is>
+          <t>SCADA/PLC, sensor maintenance</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="10" t="inlineStr">
         <is>
-          <t>S4 — Forklift Operator (greenhouse)</t>
-        </is>
-      </c>
-      <c r="B216" s="54" t="n">
+          <t>S4 — Bobcat Operator (greenhouse internal)</t>
+        </is>
+      </c>
+      <c r="B216" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C216" s="46" t="n">
-        <v>400</v>
-      </c>
-      <c r="D216" s="54" t="inlineStr">
+        <v>450</v>
+      </c>
+      <c r="D216" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7734,25 +7715,25 @@
         <f>B216*C216</f>
         <v/>
       </c>
-      <c r="F216" s="55" t="inlineStr">
-        <is>
-          <t>1.5t electric forklifts</t>
+      <c r="F216" s="54" t="inlineStr">
+        <is>
+          <t>S450, substrate + frass movement</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="10" t="inlineStr">
         <is>
-          <t>S5A — Frass Screening / Bagging Operator</t>
-        </is>
-      </c>
-      <c r="B217" s="54" t="n">
+          <t>S4 — Forklift Operator (greenhouse)</t>
+        </is>
+      </c>
+      <c r="B217" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C217" s="46" t="n">
         <v>400</v>
       </c>
-      <c r="D217" s="54" t="inlineStr">
+      <c r="D217" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7761,21 +7742,25 @@
         <f>B217*C217</f>
         <v/>
       </c>
-      <c r="F217" s="55" t="inlineStr"/>
+      <c r="F217" s="54" t="inlineStr">
+        <is>
+          <t>1.5t electric forklifts</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="10" t="inlineStr">
         <is>
-          <t>S5B — Larvae Separation Operator</t>
-        </is>
-      </c>
-      <c r="B218" s="54" t="n">
+          <t>S5A — Frass Screening / Bagging Operator</t>
+        </is>
+      </c>
+      <c r="B218" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C218" s="46" t="n">
-        <v>450</v>
-      </c>
-      <c r="D218" s="54" t="inlineStr">
+        <v>400</v>
+      </c>
+      <c r="D218" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7784,25 +7769,21 @@
         <f>B218*C218</f>
         <v/>
       </c>
-      <c r="F218" s="55" t="inlineStr">
-        <is>
-          <t>Vibrating separator + thermal</t>
-        </is>
-      </c>
+      <c r="F218" s="54" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="10" t="inlineStr">
         <is>
-          <t>S5B — Oil Press / Dryer Operator</t>
-        </is>
-      </c>
-      <c r="B219" s="54" t="n">
+          <t>S5B — Larvae Separation Operator</t>
+        </is>
+      </c>
+      <c r="B219" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C219" s="46" t="n">
-        <v>500</v>
-      </c>
-      <c r="D219" s="54" t="inlineStr">
+        <v>450</v>
+      </c>
+      <c r="D219" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7811,25 +7792,25 @@
         <f>B219*C219</f>
         <v/>
       </c>
-      <c r="F219" s="55" t="inlineStr">
-        <is>
-          <t>Screw press + belt dryer</t>
+      <c r="F219" s="54" t="inlineStr">
+        <is>
+          <t>Vibrating separator + thermal</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="10" t="inlineStr">
         <is>
-          <t>Warehouse — Forklift Operator</t>
-        </is>
-      </c>
-      <c r="B220" s="54" t="n">
+          <t>S5B — Oil Press / Dryer Operator</t>
+        </is>
+      </c>
+      <c r="B220" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C220" s="46" t="n">
-        <v>400</v>
-      </c>
-      <c r="D220" s="54" t="inlineStr">
+        <v>500</v>
+      </c>
+      <c r="D220" s="53" t="inlineStr">
         <is>
           <t>2-shift</t>
         </is>
@@ -7838,52 +7819,52 @@
         <f>B220*C220</f>
         <v/>
       </c>
-      <c r="F220" s="55" t="inlineStr">
-        <is>
-          <t>3t diesel forklift</t>
+      <c r="F220" s="54" t="inlineStr">
+        <is>
+          <t>Screw press + belt dryer</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="10" t="inlineStr">
         <is>
-          <t>Warehouse — Storeman / Inventory</t>
-        </is>
-      </c>
-      <c r="B221" s="54" t="n">
-        <v>1</v>
+          <t>Warehouse — Forklift Operator</t>
+        </is>
+      </c>
+      <c r="B221" s="53" t="n">
+        <v>2</v>
       </c>
       <c r="C221" s="46" t="n">
-        <v>450</v>
-      </c>
-      <c r="D221" s="54" t="inlineStr">
-        <is>
-          <t>day</t>
+        <v>400</v>
+      </c>
+      <c r="D221" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
         </is>
       </c>
       <c r="E221" s="22">
         <f>B221*C221</f>
         <v/>
       </c>
-      <c r="F221" s="55" t="inlineStr">
-        <is>
-          <t>Stock control, dispatch</t>
+      <c r="F221" s="54" t="inlineStr">
+        <is>
+          <t>3t diesel forklift</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="10" t="inlineStr">
         <is>
-          <t>Logistics — Flatbed Truck Driver</t>
-        </is>
-      </c>
-      <c r="B222" s="54" t="n">
+          <t>Warehouse — Storeman / Inventory</t>
+        </is>
+      </c>
+      <c r="B222" s="53" t="n">
         <v>1</v>
       </c>
       <c r="C222" s="46" t="n">
         <v>450</v>
       </c>
-      <c r="D222" s="54" t="inlineStr">
+      <c r="D222" s="53" t="inlineStr">
         <is>
           <t>day</t>
         </is>
@@ -7892,25 +7873,25 @@
         <f>B222*C222</f>
         <v/>
       </c>
-      <c r="F222" s="55" t="inlineStr">
-        <is>
-          <t>Product delivery</t>
+      <c r="F222" s="54" t="inlineStr">
+        <is>
+          <t>Stock control, dispatch</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="10" t="inlineStr">
         <is>
-          <t>Logistics — Tanker Truck Driver</t>
-        </is>
-      </c>
-      <c r="B223" s="54" t="n">
+          <t>Logistics — Flatbed Truck Driver</t>
+        </is>
+      </c>
+      <c r="B223" s="53" t="n">
         <v>1</v>
       </c>
       <c r="C223" s="46" t="n">
         <v>450</v>
       </c>
-      <c r="D223" s="54" t="inlineStr">
+      <c r="D223" s="53" t="inlineStr">
         <is>
           <t>day</t>
         </is>
@@ -7919,25 +7900,25 @@
         <f>B223*C223</f>
         <v/>
       </c>
-      <c r="F223" s="55" t="inlineStr">
-        <is>
-          <t>Water/POME</t>
+      <c r="F223" s="54" t="inlineStr">
+        <is>
+          <t>Product delivery</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="10" t="inlineStr">
         <is>
-          <t>Site Manager</t>
-        </is>
-      </c>
-      <c r="B224" s="54" t="n">
+          <t>Logistics — Tanker Truck Driver</t>
+        </is>
+      </c>
+      <c r="B224" s="53" t="n">
         <v>1</v>
       </c>
       <c r="C224" s="46" t="n">
-        <v>1500</v>
-      </c>
-      <c r="D224" s="54" t="inlineStr">
+        <v>450</v>
+      </c>
+      <c r="D224" s="53" t="inlineStr">
         <is>
           <t>day</t>
         </is>
@@ -7946,25 +7927,25 @@
         <f>B224*C224</f>
         <v/>
       </c>
-      <c r="F224" s="55" t="inlineStr">
-        <is>
-          <t>Overall plant management</t>
+      <c r="F224" s="54" t="inlineStr">
+        <is>
+          <t>Water/POME</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="10" t="inlineStr">
         <is>
-          <t>Production Supervisor (S1-S3)</t>
-        </is>
-      </c>
-      <c r="B225" s="54" t="n">
+          <t>Site Manager</t>
+        </is>
+      </c>
+      <c r="B225" s="53" t="n">
         <v>1</v>
       </c>
       <c r="C225" s="46" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D225" s="54" t="inlineStr">
+        <v>1500</v>
+      </c>
+      <c r="D225" s="53" t="inlineStr">
         <is>
           <t>day</t>
         </is>
@@ -7973,25 +7954,25 @@
         <f>B225*C225</f>
         <v/>
       </c>
-      <c r="F225" s="55" t="inlineStr">
-        <is>
-          <t>Preprocessing + treatment</t>
+      <c r="F225" s="54" t="inlineStr">
+        <is>
+          <t>Overall plant management</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="10" t="inlineStr">
         <is>
-          <t>Quality Control / Lab Technician</t>
-        </is>
-      </c>
-      <c r="B226" s="54" t="n">
-        <v>2</v>
+          <t>Production Supervisor (S1-S3)</t>
+        </is>
+      </c>
+      <c r="B226" s="53" t="n">
+        <v>1</v>
       </c>
       <c r="C226" s="46" t="n">
-        <v>650</v>
-      </c>
-      <c r="D226" s="54" t="inlineStr">
+        <v>1000</v>
+      </c>
+      <c r="D226" s="53" t="inlineStr">
         <is>
           <t>day</t>
         </is>
@@ -8000,25 +7981,25 @@
         <f>B226*C226</f>
         <v/>
       </c>
-      <c r="F226" s="55" t="inlineStr">
-        <is>
-          <t>pH, MC, ICP-OES, sampling</t>
+      <c r="F226" s="54" t="inlineStr">
+        <is>
+          <t>Preprocessing + treatment</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="10" t="inlineStr">
         <is>
-          <t>Maintenance Technician (mechanical)</t>
-        </is>
-      </c>
-      <c r="B227" s="54" t="n">
+          <t>Quality Control / Lab Technician</t>
+        </is>
+      </c>
+      <c r="B227" s="53" t="n">
         <v>2</v>
       </c>
       <c r="C227" s="46" t="n">
-        <v>600</v>
-      </c>
-      <c r="D227" s="54" t="inlineStr">
+        <v>650</v>
+      </c>
+      <c r="D227" s="53" t="inlineStr">
         <is>
           <t>day</t>
         </is>
@@ -8027,25 +8008,25 @@
         <f>B227*C227</f>
         <v/>
       </c>
-      <c r="F227" s="55" t="inlineStr">
-        <is>
-          <t>All mechanical equipment</t>
+      <c r="F227" s="54" t="inlineStr">
+        <is>
+          <t>pH, MC, ICP-OES, sampling</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="10" t="inlineStr">
         <is>
-          <t>Maintenance Technician (electrical/IoT)</t>
-        </is>
-      </c>
-      <c r="B228" s="54" t="n">
-        <v>1</v>
+          <t>Maintenance Technician (mechanical)</t>
+        </is>
+      </c>
+      <c r="B228" s="53" t="n">
+        <v>2</v>
       </c>
       <c r="C228" s="46" t="n">
-        <v>650</v>
-      </c>
-      <c r="D228" s="54" t="inlineStr">
+        <v>600</v>
+      </c>
+      <c r="D228" s="53" t="inlineStr">
         <is>
           <t>day</t>
         </is>
@@ -8054,25 +8035,25 @@
         <f>B228*C228</f>
         <v/>
       </c>
-      <c r="F228" s="55" t="inlineStr">
-        <is>
-          <t>Electrical, sensors, PLC</t>
+      <c r="F228" s="54" t="inlineStr">
+        <is>
+          <t>All mechanical equipment</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>HSE Officer</t>
-        </is>
-      </c>
-      <c r="B229" s="54" t="n">
+          <t>Maintenance Technician (electrical/IoT)</t>
+        </is>
+      </c>
+      <c r="B229" s="53" t="n">
         <v>1</v>
       </c>
       <c r="C229" s="46" t="n">
-        <v>700</v>
-      </c>
-      <c r="D229" s="54" t="inlineStr">
+        <v>650</v>
+      </c>
+      <c r="D229" s="53" t="inlineStr">
         <is>
           <t>day</t>
         </is>
@@ -8081,25 +8062,25 @@
         <f>B229*C229</f>
         <v/>
       </c>
-      <c r="F229" s="55" t="inlineStr">
-        <is>
-          <t>Safety, PPE, NaOH handling</t>
+      <c r="F229" s="54" t="inlineStr">
+        <is>
+          <t>Electrical, sensors, PLC</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="10" t="inlineStr">
         <is>
-          <t>Admin / Finance</t>
-        </is>
-      </c>
-      <c r="B230" s="54" t="n">
-        <v>2</v>
+          <t>HSE Officer</t>
+        </is>
+      </c>
+      <c r="B230" s="53" t="n">
+        <v>1</v>
       </c>
       <c r="C230" s="46" t="n">
-        <v>500</v>
-      </c>
-      <c r="D230" s="54" t="inlineStr">
+        <v>700</v>
+      </c>
+      <c r="D230" s="53" t="inlineStr">
         <is>
           <t>day</t>
         </is>
@@ -8108,371 +8089,398 @@
         <f>B230*C230</f>
         <v/>
       </c>
-      <c r="F230" s="55" t="inlineStr"/>
+      <c r="F230" s="54" t="inlineStr">
+        <is>
+          <t>Safety, PPE, NaOH handling</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="10" t="inlineStr">
         <is>
-          <t>Security (gate + night)</t>
-        </is>
-      </c>
-      <c r="B231" s="54" t="n">
-        <v>3</v>
+          <t>Admin / Finance</t>
+        </is>
+      </c>
+      <c r="B231" s="53" t="n">
+        <v>2</v>
       </c>
       <c r="C231" s="46" t="n">
-        <v>350</v>
-      </c>
-      <c r="D231" s="54" t="inlineStr">
-        <is>
-          <t>3-shift</t>
+        <v>500</v>
+      </c>
+      <c r="D231" s="53" t="inlineStr">
+        <is>
+          <t>day</t>
         </is>
       </c>
       <c r="E231" s="22">
         <f>B231*C231</f>
         <v/>
       </c>
-      <c r="F231" s="55" t="inlineStr">
-        <is>
-          <t>24/7 coverage</t>
-        </is>
-      </c>
+      <c r="F231" s="54" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="10" t="inlineStr">
         <is>
-          <t>Cleaner / General Labour</t>
-        </is>
-      </c>
-      <c r="B232" s="54" t="n">
-        <v>4</v>
+          <t>Security (gate + night)</t>
+        </is>
+      </c>
+      <c r="B232" s="53" t="n">
+        <v>3</v>
       </c>
       <c r="C232" s="46" t="n">
         <v>350</v>
       </c>
-      <c r="D232" s="54" t="inlineStr">
-        <is>
-          <t>2-shift</t>
+      <c r="D232" s="53" t="inlineStr">
+        <is>
+          <t>3-shift</t>
         </is>
       </c>
       <c r="E232" s="22">
         <f>B232*C232</f>
         <v/>
       </c>
-      <c r="F232" s="55" t="inlineStr">
+      <c r="F232" s="54" t="inlineStr">
+        <is>
+          <t>24/7 coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="10" t="inlineStr">
+        <is>
+          <t>Cleaner / General Labour</t>
+        </is>
+      </c>
+      <c r="B233" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="C233" s="46" t="n">
+        <v>350</v>
+      </c>
+      <c r="D233" s="53" t="inlineStr">
+        <is>
+          <t>2-shift</t>
+        </is>
+      </c>
+      <c r="E233" s="22">
+        <f>B233*C233</f>
+        <v/>
+      </c>
+      <c r="F233" s="54" t="inlineStr">
         <is>
           <t>Site-wide</t>
         </is>
       </c>
     </row>
-    <row r="233">
-      <c r="A233" s="15" t="inlineStr">
+    <row r="234">
+      <c r="A234" s="15" t="inlineStr">
         <is>
           <t>TOTAL STAFFING</t>
         </is>
       </c>
-      <c r="B233" s="56">
-        <f>SUM(B198:B232)</f>
-        <v/>
-      </c>
-      <c r="E233" s="51">
-        <f>SUM(E198:E232)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" s="7" t="inlineStr">
+      <c r="B234" s="55">
+        <f>SUM(B199:B233)</f>
+        <v/>
+      </c>
+      <c r="E234" s="51">
+        <f>SUM(E199:E233)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="7" t="inlineStr">
         <is>
           <t>ANNUAL LABOUR COST (x12 months)</t>
         </is>
       </c>
-      <c r="E234" s="22">
-        <f>E233*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" s="3" t="inlineStr">
+      <c r="E235" s="22">
+        <f>E234*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="3" t="inlineStr">
         <is>
           <t>TOTAL CAPEX SUMMARY</t>
         </is>
       </c>
-      <c r="B236" s="3" t="n"/>
-      <c r="C236" s="3" t="n"/>
-    </row>
-    <row r="237">
-      <c r="A237" s="38" t="inlineStr">
+      <c r="B237" s="3" t="n"/>
+      <c r="C237" s="3" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="38" t="inlineStr">
         <is>
           <t>TOTAL CAPEX</t>
         </is>
       </c>
-      <c r="B237" s="51">
-        <f>IFERROR(SUM(B5:B236),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" s="3" t="inlineStr">
+      <c r="B238" s="51">
+        <f>IFERROR(SUM(B5:B237),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="3" t="inlineStr">
         <is>
           <t>MONTHLY OPERATING EXPENDITURE (OPEX)</t>
         </is>
       </c>
-      <c r="B239" s="3" t="n"/>
-      <c r="C239" s="3" t="n"/>
-      <c r="D239" s="3" t="n"/>
-    </row>
-    <row r="240">
-      <c r="A240" s="9" t="inlineStr">
+      <c r="B240" s="3" t="n"/>
+      <c r="C240" s="3" t="n"/>
+      <c r="D240" s="3" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="9" t="inlineStr">
         <is>
           <t>Cost Item</t>
         </is>
       </c>
-      <c r="B240" s="9" t="inlineStr">
+      <c r="B241" s="9" t="inlineStr">
         <is>
           <t>Monthly Cost (USD)</t>
         </is>
       </c>
-      <c r="C240" s="9" t="inlineStr">
+      <c r="C241" s="9" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" s="10" t="inlineStr">
-        <is>
-          <t>Chemical Treatment</t>
-        </is>
-      </c>
-      <c r="B241" s="22">
-        <f>IFERROR(S2_Chemical_Treatment!B33,0)</f>
-        <v/>
-      </c>
-      <c r="C241" s="2" t="inlineStr">
-        <is>
-          <t>From Stage 2</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="10" t="inlineStr">
         <is>
-          <t>Biological Treatment</t>
+          <t>Chemical Treatment</t>
         </is>
       </c>
       <c r="B242" s="22">
-        <f>IFERROR(S3_Biological_Treatment!B33,0)</f>
+        <f>IFERROR(S2_Chemical_Treatment!B33,0)</f>
         <v/>
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>From Stage 3</t>
+          <t>From Stage 2</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="10" t="inlineStr">
         <is>
-          <t>BSF Neonates</t>
+          <t>Biological Treatment</t>
         </is>
       </c>
       <c r="B243" s="22">
-        <f>IFERROR(S4_BSF_Rearing!B8,0)</f>
+        <f>IFERROR(S3_Biological_Treatment!B33,0)</f>
         <v/>
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>From Stage 4</t>
+          <t>From Stage 3</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="10" t="inlineStr">
         <is>
-          <t>Processing (S5B)</t>
+          <t>BSF Neonates</t>
         </is>
       </c>
       <c r="B244" s="22">
-        <f>IFERROR(S5B_BSF_Extraction!B29,0)</f>
+        <f>IFERROR(S4_BSF_Rearing!B8,0)</f>
         <v/>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>From Stage 5B</t>
+          <t>From Stage 4</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="10" t="inlineStr">
         <is>
-          <t>Energy / Utilities</t>
+          <t>Processing (S5B)</t>
         </is>
       </c>
       <c r="B245" s="22">
-        <f>IFERROR(S1_Preprocessing!B30,0)</f>
+        <f>IFERROR(S5B_BSF_Extraction!B29,0)</f>
         <v/>
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>From Stage 1</t>
+          <t>From Stage 5B</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="10" t="inlineStr">
         <is>
-          <t>Labour (full staffing)</t>
+          <t>Energy / Utilities</t>
         </is>
       </c>
       <c r="B246" s="22">
-        <f>E233</f>
+        <f>IFERROR(S1_Preprocessing!B30,0)</f>
         <v/>
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>67 staff — see staffing section row 233</t>
+          <t>From Stage 1</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="10" t="inlineStr">
         <is>
-          <t>Maintenance (2% CAPEX/month)</t>
+          <t>Labour (full staffing)</t>
         </is>
       </c>
       <c r="B247" s="22">
-        <f>IFERROR(B237*0.02/12,0)</f>
+        <f>E234</f>
         <v/>
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>Industry standard</t>
+          <t>67 staff — see staffing section row 234</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="10" t="inlineStr">
         <is>
-          <t>Quality Control / Lab</t>
-        </is>
-      </c>
-      <c r="B248" s="46" t="n">
-        <v>2000</v>
+          <t>Maintenance (2% CAPEX/month)</t>
+        </is>
+      </c>
+      <c r="B248" s="22">
+        <f>IFERROR(B238*0.02/12,0)</f>
+        <v/>
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>Monthly QC testing</t>
+          <t>Industry standard</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="10" t="inlineStr">
         <is>
+          <t>Quality Control / Lab</t>
+        </is>
+      </c>
+      <c r="B249" s="46" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>Monthly QC testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="10" t="inlineStr">
+        <is>
           <t>Transport / Logistics</t>
         </is>
       </c>
-      <c r="B249" s="46" t="n">
+      <c r="B250" s="46" t="n">
         <v>3000</v>
       </c>
-      <c r="C249" s="2" t="inlineStr">
+      <c r="C250" s="2" t="inlineStr">
         <is>
           <t>Product distribution</t>
         </is>
       </c>
     </row>
-    <row r="250">
-      <c r="A250" s="38" t="inlineStr">
+    <row r="251">
+      <c r="A251" s="38" t="inlineStr">
         <is>
           <t>TOTAL MONTHLY OPEX</t>
         </is>
       </c>
-      <c r="B250" s="52">
-        <f>IFERROR(SUM(B241:B249),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" s="3" t="inlineStr">
+      <c r="B251" s="52">
+        <f>IFERROR(SUM(B242:B250),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="3" t="inlineStr">
         <is>
           <t>PAYBACK &amp; NPV ANALYSIS</t>
         </is>
       </c>
-      <c r="B252" s="3" t="n"/>
-      <c r="C252" s="3" t="n"/>
-      <c r="D252" s="3" t="n"/>
-    </row>
-    <row r="253">
-      <c r="A253" s="4" t="inlineStr">
-        <is>
-          <t>Total CAPEX</t>
-        </is>
-      </c>
-      <c r="B253" s="22">
-        <f>B237</f>
-        <v/>
-      </c>
+      <c r="B253" s="3" t="n"/>
+      <c r="C253" s="3" t="n"/>
+      <c r="D253" s="3" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="4" t="inlineStr">
         <is>
+          <t>Total CAPEX</t>
+        </is>
+      </c>
+      <c r="B254" s="22">
+        <f>B238</f>
+        <v/>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="4" t="inlineStr">
+        <is>
           <t>Monthly Gross Profit</t>
         </is>
       </c>
-      <c r="B254" s="22">
-        <f>IFERROR(Summary_Dashboard!B24-B250,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" s="38" t="inlineStr">
+      <c r="B255" s="22">
+        <f>IFERROR(Summary_Dashboard!B24-B251,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="38" t="inlineStr">
         <is>
           <t>Payback Period (months)</t>
         </is>
       </c>
-      <c r="B255" s="42">
-        <f>IFERROR(B253/B254,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" s="4" t="inlineStr">
+      <c r="B256" s="42">
+        <f>IFERROR(B254/B255,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="4" t="inlineStr">
         <is>
           <t>Payback Period (years)</t>
         </is>
       </c>
-      <c r="B256" s="13">
-        <f>IFERROR(B255/12,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" s="4" t="inlineStr">
-        <is>
-          <t>IRR Discount Rate (user-adjustable)</t>
-        </is>
-      </c>
-      <c r="B258" s="57" t="n">
-        <v>0.12</v>
+      <c r="B257" s="13">
+        <f>IFERROR(B256/12,0)</f>
+        <v/>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
         <is>
+          <t>IRR Discount Rate (user-adjustable)</t>
+        </is>
+      </c>
+      <c r="B259" s="56" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="4" t="inlineStr">
+        <is>
           <t>Annual Net Cash Flow</t>
         </is>
       </c>
-      <c r="B259" s="22">
-        <f>IFERROR(B254*12,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" s="7" t="inlineStr">
+      <c r="B260" s="22">
+        <f>IFERROR(B255*12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="7" t="inlineStr">
         <is>
           <t>5-Year NPV (simple estimate)</t>
         </is>
       </c>
-      <c r="B260" s="30">
-        <f>IFERROR(B259/(1+B258)^1+B259/(1+B258)^2+B259/(1+B258)^3+B259/(1+B258)^4+B259/(1+B258)^5-B253,0)</f>
+      <c r="B261" s="30">
+        <f>IFERROR(B260/(1+B259)^1+B260/(1+B259)^2+B260/(1+B259)^3+B260/(1+B259)^4+B260/(1+B259)^5-B254,0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add development markups: PE/Fixer 20%, Local EPC 15%, PRI 2% annual
- Process Engineer/Fixer @ 20% on equipment CAPEX (NOT on EPC building)
- Local EPC @ 15% on total (equipment + building)
- Political Risk Insurance @ 2% p.a. added to OPEX (monthly provision)
- Equipment subtotal formula excludes Process Building EPC to avoid double markup

https://claude.ai/code/session_01WZKNxbjsTJxtui6XGx7d89
</commit_message>
<xml_diff>
--- a/CFI_Master_Excel.xlsx
+++ b/CFI_Master_Excel.xlsx
@@ -4549,7 +4549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F261"/>
+  <dimension ref="A1:F269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -8201,286 +8201,387 @@
     <row r="237">
       <c r="A237" s="3" t="inlineStr">
         <is>
-          <t>TOTAL CAPEX SUMMARY</t>
+          <t>DEVELOPMENT &amp; INSTALLATION MARKUPS</t>
         </is>
       </c>
       <c r="B237" s="3" t="n"/>
       <c r="C237" s="3" t="n"/>
     </row>
     <row r="238">
-      <c r="A238" s="38" t="inlineStr">
-        <is>
-          <t>TOTAL CAPEX</t>
-        </is>
-      </c>
-      <c r="B238" s="51">
-        <f>IFERROR(SUM(B5:B237),0)</f>
-        <v/>
+      <c r="A238" s="9" t="inlineStr">
+        <is>
+          <t>Equipment / Item</t>
+        </is>
+      </c>
+      <c r="B238" s="9" t="inlineStr">
+        <is>
+          <t>Estimated Cost (USD)</t>
+        </is>
+      </c>
+      <c r="C238" s="9" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="7" t="inlineStr">
+        <is>
+          <t>Equipment CAPEX Subtotal (excl. Process Building EPC)</t>
+        </is>
+      </c>
+      <c r="B239" s="22">
+        <f>IFERROR(SUM(B5:B236)-SUM(B97:B107),0)</f>
+        <v/>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>Base for PE/Fixer</t>
+        </is>
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="3" t="inlineStr">
+      <c r="A240" s="10" t="inlineStr">
+        <is>
+          <t>Process Engineer / Fixer @ 20% (on equipment, NOT on EPC)</t>
+        </is>
+      </c>
+      <c r="B240" s="22">
+        <f>IFERROR(B239*0.20,0)</f>
+        <v/>
+      </c>
+      <c r="C240" s="10" t="inlineStr">
+        <is>
+          <t>Markup</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="10" t="inlineStr">
+        <is>
+          <t>Local EPC @ 15%</t>
+        </is>
+      </c>
+      <c r="B241" s="22">
+        <f>IFERROR((B239+SUM(B97:B107))*0.15,0)</f>
+        <v/>
+      </c>
+      <c r="C241" s="10" t="inlineStr">
+        <is>
+          <t>Markup</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="7" t="inlineStr">
+        <is>
+          <t>Markups Subtotal</t>
+        </is>
+      </c>
+      <c r="B242" s="22">
+        <f>SUM(B240:B241)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL CAPEX SUMMARY</t>
+        </is>
+      </c>
+      <c r="B244" s="3" t="n"/>
+      <c r="C244" s="3" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="38" t="inlineStr">
+        <is>
+          <t>TOTAL CAPEX (all equipment + building + markups)</t>
+        </is>
+      </c>
+      <c r="B245" s="51">
+        <f>IFERROR(SUM(B5:B244),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="3" t="inlineStr">
         <is>
           <t>MONTHLY OPERATING EXPENDITURE (OPEX)</t>
         </is>
       </c>
-      <c r="B240" s="3" t="n"/>
-      <c r="C240" s="3" t="n"/>
-      <c r="D240" s="3" t="n"/>
-    </row>
-    <row r="241">
-      <c r="A241" s="9" t="inlineStr">
+      <c r="B247" s="3" t="n"/>
+      <c r="C247" s="3" t="n"/>
+      <c r="D247" s="3" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="9" t="inlineStr">
         <is>
           <t>Cost Item</t>
         </is>
       </c>
-      <c r="B241" s="9" t="inlineStr">
+      <c r="B248" s="9" t="inlineStr">
         <is>
           <t>Monthly Cost (USD)</t>
         </is>
       </c>
-      <c r="C241" s="9" t="inlineStr">
+      <c r="C248" s="9" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" s="10" t="inlineStr">
-        <is>
-          <t>Chemical Treatment</t>
-        </is>
-      </c>
-      <c r="B242" s="22">
-        <f>IFERROR(S2_Chemical_Treatment!B33,0)</f>
-        <v/>
-      </c>
-      <c r="C242" s="2" t="inlineStr">
-        <is>
-          <t>From Stage 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" s="10" t="inlineStr">
-        <is>
-          <t>Biological Treatment</t>
-        </is>
-      </c>
-      <c r="B243" s="22">
-        <f>IFERROR(S3_Biological_Treatment!B33,0)</f>
-        <v/>
-      </c>
-      <c r="C243" s="2" t="inlineStr">
-        <is>
-          <t>From Stage 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" s="10" t="inlineStr">
-        <is>
-          <t>BSF Neonates</t>
-        </is>
-      </c>
-      <c r="B244" s="22">
-        <f>IFERROR(S4_BSF_Rearing!B8,0)</f>
-        <v/>
-      </c>
-      <c r="C244" s="2" t="inlineStr">
-        <is>
-          <t>From Stage 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" s="10" t="inlineStr">
-        <is>
-          <t>Processing (S5B)</t>
-        </is>
-      </c>
-      <c r="B245" s="22">
-        <f>IFERROR(S5B_BSF_Extraction!B29,0)</f>
-        <v/>
-      </c>
-      <c r="C245" s="2" t="inlineStr">
-        <is>
-          <t>From Stage 5B</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" s="10" t="inlineStr">
-        <is>
-          <t>Energy / Utilities</t>
-        </is>
-      </c>
-      <c r="B246" s="22">
-        <f>IFERROR(S1_Preprocessing!B30,0)</f>
-        <v/>
-      </c>
-      <c r="C246" s="2" t="inlineStr">
-        <is>
-          <t>From Stage 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" s="10" t="inlineStr">
-        <is>
-          <t>Labour (full staffing)</t>
-        </is>
-      </c>
-      <c r="B247" s="22">
-        <f>E234</f>
-        <v/>
-      </c>
-      <c r="C247" s="2" t="inlineStr">
-        <is>
-          <t>67 staff — see staffing section row 234</t>
-        </is>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" s="10" t="inlineStr">
-        <is>
-          <t>Maintenance (2% CAPEX/month)</t>
-        </is>
-      </c>
-      <c r="B248" s="22">
-        <f>IFERROR(B238*0.02/12,0)</f>
-        <v/>
-      </c>
-      <c r="C248" s="2" t="inlineStr">
-        <is>
-          <t>Industry standard</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="10" t="inlineStr">
         <is>
-          <t>Quality Control / Lab</t>
-        </is>
-      </c>
-      <c r="B249" s="46" t="n">
-        <v>2000</v>
+          <t>Chemical Treatment</t>
+        </is>
+      </c>
+      <c r="B249" s="22">
+        <f>IFERROR(S2_Chemical_Treatment!B33,0)</f>
+        <v/>
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>Monthly QC testing</t>
+          <t>From Stage 2</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="10" t="inlineStr">
         <is>
+          <t>Biological Treatment</t>
+        </is>
+      </c>
+      <c r="B250" s="22">
+        <f>IFERROR(S3_Biological_Treatment!B33,0)</f>
+        <v/>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>From Stage 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="10" t="inlineStr">
+        <is>
+          <t>BSF Neonates</t>
+        </is>
+      </c>
+      <c r="B251" s="22">
+        <f>IFERROR(S4_BSF_Rearing!B8,0)</f>
+        <v/>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>From Stage 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="10" t="inlineStr">
+        <is>
+          <t>Processing (S5B)</t>
+        </is>
+      </c>
+      <c r="B252" s="22">
+        <f>IFERROR(S5B_BSF_Extraction!B29,0)</f>
+        <v/>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>From Stage 5B</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="10" t="inlineStr">
+        <is>
+          <t>Energy / Utilities</t>
+        </is>
+      </c>
+      <c r="B253" s="22">
+        <f>IFERROR(S1_Preprocessing!B30,0)</f>
+        <v/>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>From Stage 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="10" t="inlineStr">
+        <is>
+          <t>Labour (full staffing)</t>
+        </is>
+      </c>
+      <c r="B254" s="22">
+        <f>E234</f>
+        <v/>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>67 staff — see staffing section row 234</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="10" t="inlineStr">
+        <is>
+          <t>Maintenance (2% CAPEX/month)</t>
+        </is>
+      </c>
+      <c r="B255" s="22">
+        <f>IFERROR(B245*0.02/12,0)</f>
+        <v/>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>Industry standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="10" t="inlineStr">
+        <is>
+          <t>Political Risk Insurance @ 2% p.a.</t>
+        </is>
+      </c>
+      <c r="B256" s="22">
+        <f>IFERROR(B245*0.02/12,0)</f>
+        <v/>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>2% annual on total CAPEX, monthly provision</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="10" t="inlineStr">
+        <is>
+          <t>Quality Control / Lab</t>
+        </is>
+      </c>
+      <c r="B257" s="46" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>Monthly QC testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="10" t="inlineStr">
+        <is>
           <t>Transport / Logistics</t>
         </is>
       </c>
-      <c r="B250" s="46" t="n">
+      <c r="B258" s="46" t="n">
         <v>3000</v>
       </c>
-      <c r="C250" s="2" t="inlineStr">
+      <c r="C258" s="2" t="inlineStr">
         <is>
           <t>Product distribution</t>
         </is>
       </c>
     </row>
-    <row r="251">
-      <c r="A251" s="38" t="inlineStr">
+    <row r="259">
+      <c r="A259" s="38" t="inlineStr">
         <is>
           <t>TOTAL MONTHLY OPEX</t>
         </is>
       </c>
-      <c r="B251" s="52">
-        <f>IFERROR(SUM(B242:B250),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" s="3" t="inlineStr">
+      <c r="B259" s="52">
+        <f>IFERROR(SUM(B249:B258),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="3" t="inlineStr">
         <is>
           <t>PAYBACK &amp; NPV ANALYSIS</t>
         </is>
       </c>
-      <c r="B253" s="3" t="n"/>
-      <c r="C253" s="3" t="n"/>
-      <c r="D253" s="3" t="n"/>
-    </row>
-    <row r="254">
-      <c r="A254" s="4" t="inlineStr">
+      <c r="B261" s="3" t="n"/>
+      <c r="C261" s="3" t="n"/>
+      <c r="D261" s="3" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="4" t="inlineStr">
         <is>
           <t>Total CAPEX</t>
         </is>
       </c>
-      <c r="B254" s="22">
-        <f>B238</f>
-        <v/>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" s="4" t="inlineStr">
+      <c r="B262" s="22">
+        <f>B245</f>
+        <v/>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="4" t="inlineStr">
         <is>
           <t>Monthly Gross Profit</t>
         </is>
       </c>
-      <c r="B255" s="22">
-        <f>IFERROR(Summary_Dashboard!B24-B251,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" s="38" t="inlineStr">
+      <c r="B263" s="22">
+        <f>IFERROR(Summary_Dashboard!B24-B259,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="38" t="inlineStr">
         <is>
           <t>Payback Period (months)</t>
         </is>
       </c>
-      <c r="B256" s="42">
-        <f>IFERROR(B254/B255,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" s="4" t="inlineStr">
+      <c r="B264" s="42">
+        <f>IFERROR(B262/B263,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="4" t="inlineStr">
         <is>
           <t>Payback Period (years)</t>
         </is>
       </c>
-      <c r="B257" s="13">
-        <f>IFERROR(B256/12,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" s="4" t="inlineStr">
+      <c r="B265" s="13">
+        <f>IFERROR(B264/12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="4" t="inlineStr">
         <is>
           <t>IRR Discount Rate (user-adjustable)</t>
         </is>
       </c>
-      <c r="B259" s="56" t="n">
+      <c r="B267" s="56" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="260">
-      <c r="A260" s="4" t="inlineStr">
+    <row r="268">
+      <c r="A268" s="4" t="inlineStr">
         <is>
           <t>Annual Net Cash Flow</t>
         </is>
       </c>
-      <c r="B260" s="22">
-        <f>IFERROR(B255*12,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" s="7" t="inlineStr">
+      <c r="B268" s="22">
+        <f>IFERROR(B263*12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="7" t="inlineStr">
         <is>
           <t>5-Year NPV (simple estimate)</t>
         </is>
       </c>
-      <c r="B261" s="30">
-        <f>IFERROR(B260/(1+B259)^1+B260/(1+B259)^2+B260/(1+B259)^3+B260/(1+B259)^4+B260/(1+B259)^5-B254,0)</f>
+      <c r="B269" s="30">
+        <f>IFERROR(B268/(1+B267)^1+B268/(1+B267)^2+B268/(1+B267)^3+B268/(1+B267)^4+B268/(1+B267)^5-B262,0)</f>
         <v/>
       </c>
     </row>

</xml_diff>